<commit_message>
Paper v2 en la voz de Jesús (12 capítulos, 35 páginas); hoja Embudo con costo, ganancia y techo por paso; Excel, generador y skill regenerados
- Paper reescrito en primera persona, con cada número derivado paso a paso: cadena, techo (= costo + ganancia + fijos repartidos), termómetro del CPL, diagnóstico en orden, acelerador y freno (rendimientos decrecientes, guardarraíl, escalones, farmeo, ciclo de vida), palancas (escenarios y sensibilidad), caja (facturado vs cash, proyección, caja necesaria), rutina, errores, uso de los Excel.
- Hoja Embudo: se quita '% que se pierde'; columnas costo → ganancia → techo con nombres llanos y fila de comprobación.
- calculadora.py y SKILL.md alineados con las columnas nuevas; zip de la skill regenerado.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/01_Modelo_Financiero_Embudo_Low_Ticket_Bumps_Upsells.xlsx
+++ b/excel/01_Modelo_Financiero_Embudo_Low_Ticket_Bumps_Upsells.xlsx
@@ -169,8 +169,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -959,7 +959,7 @@
           <t>&lt;0,20</t>
         </is>
       </c>
-      <c r="G6" s="17">
+      <c r="G6" s="18">
         <f>'Modelo'!$C$7</f>
         <v/>
       </c>
@@ -995,7 +995,7 @@
           <t>&gt;5 %</t>
         </is>
       </c>
-      <c r="G7" s="18">
+      <c r="G7" s="17">
         <f>'Supuestos'!$C$12</f>
         <v/>
       </c>
@@ -1031,7 +1031,7 @@
           <t>&gt;30 %</t>
         </is>
       </c>
-      <c r="G8" s="18">
+      <c r="G8" s="17">
         <f>'Supuestos'!$C$13</f>
         <v/>
       </c>
@@ -1103,7 +1103,7 @@
           <t>&gt;35 %</t>
         </is>
       </c>
-      <c r="G10" s="18">
+      <c r="G10" s="17">
         <f>'Supuestos'!$C$18</f>
         <v/>
       </c>
@@ -1139,7 +1139,7 @@
           <t>&gt;14 %</t>
         </is>
       </c>
-      <c r="G11" s="18">
+      <c r="G11" s="17">
         <f>'Supuestos'!$C$22</f>
         <v/>
       </c>
@@ -1175,7 +1175,7 @@
           <t>&gt;4 %</t>
         </is>
       </c>
-      <c r="G12" s="18">
+      <c r="G12" s="17">
         <f>'Supuestos'!$C$30</f>
         <v/>
       </c>
@@ -1283,7 +1283,7 @@
           <t>&lt;4 %</t>
         </is>
       </c>
-      <c r="G15" s="18">
+      <c r="G15" s="17">
         <f>'Supuestos'!$C$35</f>
         <v/>
       </c>
@@ -2046,7 +2046,7 @@
         </is>
       </c>
       <c r="C7" s="35">
-        <f>IF(ISERROR(SUM('Embudo'!C5:I60)),"REVISAR","OK")</f>
+        <f>IF(ISERROR(SUM('Embudo'!C5:H60)),"REVISAR","OK")</f>
         <v/>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -2798,7 +2798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J24"/>
+  <dimension ref="B2:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -2806,24 +2806,23 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Embudo: todos los pasos, cuántos, qué porcentaje pasa y cuánto cuesta cada uno</t>
+          <t>Embudo: todos los pasos, cuántos pasan y, por cada uno, qué pagás, qué te queda y hasta cuánto podrías pagar</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Cada fila es un paso del embudo en orden. '% que pasa' compara con el paso anterior (o con el que dice la nota). El costo por paso es inversión ÷ cantidad; el techo por paso es lo máximo que podrías pagar por él si lo demás se mantiene. Los pasos sin costo propio ya se pagaron con el CPA: mejoran el AOV.</t>
+          <t>Cada fila es un paso del embudo en orden. '% que pasa' compara con el paso anterior (o con el que dice la nota). Tres números por paso: lo que pagás hoy por cada uno (inversión ÷ cantidad), lo que te queda por cada uno (ganancia ÷ cantidad) y lo máximo que podrías pagar (el techo: lo que cada uno genera en cash neto). Techo = costo + ganancia + fijos repartidos.</t>
         </is>
       </c>
     </row>
@@ -2845,30 +2844,25 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>% que se pierde</t>
+          <t>% acumulado</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>% acumulado</t>
+          <t>Costo por paso (pagás hoy)</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Costo por paso</t>
+          <t>Ganancia por paso (te queda)</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Techo por paso</t>
+          <t>Techo por paso (máximo a pagar)</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>Ganancia por paso</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>Qué se paga acá / cómo se lee</t>
         </is>
@@ -2889,28 +2883,23 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F6" s="16">
+      <c r="E6" s="16">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$8/'Modelo'!$C$8)</f>
         <v/>
       </c>
+      <c r="F6" s="11">
+        <f>IF('Modelo'!$C$8=0,0,'Supuestos'!$C$8*1/'Modelo'!$C$8)</f>
+        <v/>
+      </c>
       <c r="G6" s="11">
-        <f>IF('Modelo'!$C$8=0,0,'Supuestos'!$C$8*1/'Modelo'!$C$8)</f>
-        <v/>
-      </c>
-      <c r="H6" s="17">
+        <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$41*1/'Modelo'!$C$8)</f>
+        <v/>
+      </c>
+      <c r="H6" s="11">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$47*'Modelo'!$C$8*1/'Modelo'!$C$8)</f>
         <v/>
       </c>
-      <c r="I6" s="11">
-        <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$41*1/'Modelo'!$C$8)</f>
-        <v/>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>La unidad que compra la pauta. Costo por visita.</t>
         </is>
@@ -2926,31 +2915,27 @@
         <f>'Modelo'!$C$9</f>
         <v/>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="17">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$9/'Modelo'!$C$8)</f>
         <v/>
       </c>
-      <c r="E7" s="18">
-        <f>IF('Modelo'!$C$8=0,0,1-'Modelo'!$C$9/'Modelo'!$C$8)</f>
-        <v/>
-      </c>
-      <c r="F7" s="16">
+      <c r="E7" s="16">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$9/'Modelo'!$C$8)</f>
         <v/>
       </c>
+      <c r="F7" s="11">
+        <f>IF('Modelo'!$C$9=0,0,'Supuestos'!$C$8*1/'Modelo'!$C$9)</f>
+        <v/>
+      </c>
       <c r="G7" s="11">
-        <f>IF('Modelo'!$C$9=0,0,'Supuestos'!$C$8*1/'Modelo'!$C$9)</f>
-        <v/>
-      </c>
-      <c r="H7" s="17">
+        <f>IF('Modelo'!$C$9=0,0,'Modelo'!$C$41*1/'Modelo'!$C$9)</f>
+        <v/>
+      </c>
+      <c r="H7" s="11">
         <f>IF('Modelo'!$C$9=0,0,'Modelo'!$C$47*'Modelo'!$C$8*1/'Modelo'!$C$9)</f>
         <v/>
       </c>
-      <c r="I7" s="11">
-        <f>IF('Modelo'!$C$9=0,0,'Modelo'!$C$41*1/'Modelo'!$C$9)</f>
-        <v/>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>Costo por checkout. Si se pierde mucho acá, es la VSL.</t>
         </is>
@@ -2966,31 +2951,27 @@
         <f>'Modelo'!$C$10</f>
         <v/>
       </c>
-      <c r="D8" s="18">
+      <c r="D8" s="17">
         <f>IF('Modelo'!$C$9=0,0,'Modelo'!$C$10/'Modelo'!$C$9)</f>
         <v/>
       </c>
-      <c r="E8" s="18">
-        <f>IF('Modelo'!$C$9=0,0,1-'Modelo'!$C$10/'Modelo'!$C$9)</f>
-        <v/>
-      </c>
-      <c r="F8" s="16">
+      <c r="E8" s="16">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$10/'Modelo'!$C$8)</f>
         <v/>
       </c>
+      <c r="F8" s="11">
+        <f>IF('Modelo'!$C$10=0,0,'Supuestos'!$C$8*1/'Modelo'!$C$10)</f>
+        <v/>
+      </c>
       <c r="G8" s="11">
-        <f>IF('Modelo'!$C$10=0,0,'Supuestos'!$C$8*1/'Modelo'!$C$10)</f>
-        <v/>
-      </c>
-      <c r="H8" s="17">
+        <f>IF('Modelo'!$C$10=0,0,'Modelo'!$C$41*1/'Modelo'!$C$10)</f>
+        <v/>
+      </c>
+      <c r="H8" s="11">
         <f>IF('Modelo'!$C$10=0,0,'Modelo'!$C$47*'Modelo'!$C$8*1/'Modelo'!$C$10)</f>
         <v/>
       </c>
-      <c r="I8" s="11">
-        <f>IF('Modelo'!$C$10=0,0,'Modelo'!$C$41*1/'Modelo'!$C$10)</f>
-        <v/>
-      </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>CPA: costo por comprador. Si se pierde mucho acá, es el checkout o la oferta.</t>
         </is>
@@ -3006,21 +2987,22 @@
         <f>'Modelo'!$C$15</f>
         <v/>
       </c>
-      <c r="D9" s="18">
+      <c r="D9" s="17">
         <f>IF('Modelo'!$C$10=0,0,'Modelo'!$C$15/'Modelo'!$C$10)</f>
         <v/>
       </c>
-      <c r="E9" s="18">
-        <f>IF('Modelo'!$C$10=0,0,1-'Modelo'!$C$15/'Modelo'!$C$10)</f>
-        <v/>
-      </c>
-      <c r="F9" s="16">
+      <c r="E9" s="16">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$15/'Modelo'!$C$8)</f>
         <v/>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>sin costo propio</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>sin costo propio</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -3028,12 +3010,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>Sobre compradores del principal. Se pagó con el CPA; suma al AOV.</t>
         </is>
@@ -3049,21 +3026,22 @@
         <f>'Modelo'!$C$17</f>
         <v/>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="17">
         <f>IF('Modelo'!$C$10=0,0,'Modelo'!$C$17/'Modelo'!$C$10)</f>
         <v/>
       </c>
-      <c r="E10" s="18">
-        <f>IF('Modelo'!$C$10=0,0,1-'Modelo'!$C$17/'Modelo'!$C$10)</f>
-        <v/>
-      </c>
-      <c r="F10" s="16">
+      <c r="E10" s="16">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$17/'Modelo'!$C$8)</f>
         <v/>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>sin costo propio</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>sin costo propio</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -3071,12 +3049,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Sobre compradores del principal.</t>
         </is>
@@ -3092,21 +3065,22 @@
         <f>'Modelo'!$C$19</f>
         <v/>
       </c>
-      <c r="D11" s="18">
+      <c r="D11" s="17">
         <f>IF('Modelo'!$C$10=0,0,'Modelo'!$C$19/'Modelo'!$C$10)</f>
         <v/>
       </c>
-      <c r="E11" s="18">
-        <f>IF('Modelo'!$C$10=0,0,1-'Modelo'!$C$19/'Modelo'!$C$10)</f>
-        <v/>
-      </c>
-      <c r="F11" s="16">
+      <c r="E11" s="16">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$19/'Modelo'!$C$8)</f>
         <v/>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>sin costo propio</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>sin costo propio</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -3114,12 +3088,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>Página 1 después del pago.</t>
         </is>
@@ -3135,21 +3104,22 @@
         <f>'Modelo'!$C$21</f>
         <v/>
       </c>
-      <c r="D12" s="18">
+      <c r="D12" s="17">
         <f>IF('Modelo'!$C$10=0,0,'Modelo'!$C$21/'Modelo'!$C$10)</f>
         <v/>
       </c>
-      <c r="E12" s="18">
-        <f>IF('Modelo'!$C$10=0,0,1-'Modelo'!$C$21/'Modelo'!$C$10)</f>
-        <v/>
-      </c>
-      <c r="F12" s="16">
+      <c r="E12" s="16">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$21/'Modelo'!$C$8)</f>
         <v/>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>sin costo propio</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>sin costo propio</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -3157,12 +3127,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>Página 2 (downsell de la OTO 1).</t>
         </is>
@@ -3178,21 +3143,22 @@
         <f>'Modelo'!$C$23</f>
         <v/>
       </c>
-      <c r="D13" s="18">
+      <c r="D13" s="17">
         <f>IF('Modelo'!$C$10=0,0,'Modelo'!$C$23/'Modelo'!$C$10)</f>
         <v/>
       </c>
-      <c r="E13" s="18">
-        <f>IF('Modelo'!$C$10=0,0,1-'Modelo'!$C$23/'Modelo'!$C$10)</f>
-        <v/>
-      </c>
-      <c r="F13" s="16">
+      <c r="E13" s="16">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$23/'Modelo'!$C$8)</f>
         <v/>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>sin costo propio</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>sin costo propio</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -3200,12 +3166,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>Página 3.</t>
         </is>
@@ -3221,21 +3182,22 @@
         <f>'Modelo'!$C$25</f>
         <v/>
       </c>
-      <c r="D14" s="18">
+      <c r="D14" s="17">
         <f>IF('Modelo'!$C$10=0,0,'Modelo'!$C$25/'Modelo'!$C$10)</f>
         <v/>
       </c>
-      <c r="E14" s="18">
-        <f>IF('Modelo'!$C$10=0,0,1-'Modelo'!$C$25/'Modelo'!$C$10)</f>
-        <v/>
-      </c>
-      <c r="F14" s="16">
+      <c r="E14" s="16">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$25/'Modelo'!$C$8)</f>
         <v/>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>sin costo propio</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>sin costo propio</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -3243,12 +3205,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>Página 4.</t>
         </is>
@@ -3264,21 +3221,22 @@
         <f>'Modelo'!$C$27</f>
         <v/>
       </c>
-      <c r="D15" s="18">
+      <c r="D15" s="17">
         <f>IF('Modelo'!$C$10=0,0,'Modelo'!$C$27/'Modelo'!$C$10)</f>
         <v/>
       </c>
-      <c r="E15" s="18">
-        <f>IF('Modelo'!$C$10=0,0,1-'Modelo'!$C$27/'Modelo'!$C$10)</f>
-        <v/>
-      </c>
-      <c r="F15" s="16">
+      <c r="E15" s="16">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$27/'Modelo'!$C$8)</f>
         <v/>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>sin costo propio</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>sin costo propio</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -3286,12 +3244,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>Sobre compradores del principal. El AOV neto resultante contra el CPA es lo que decide el embudo.</t>
         </is>
@@ -3300,53 +3253,70 @@
     <row r="17">
       <c r="B17" s="3" t="inlineStr">
         <is>
+          <t>Comprobalo con la fila de la unidad: costo + ganancia + fijos repartidos = techo</t>
+        </is>
+      </c>
+      <c r="F17" s="18">
+        <f>F6</f>
+        <v/>
+      </c>
+      <c r="G17" s="18">
+        <f>G6</f>
+        <v/>
+      </c>
+      <c r="H17" s="11">
+        <f>F6+G6+'Supuestos'!$C$37/'Modelo'!$C$8</f>
+        <v/>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Techo = costo + ganancia + fijos ÷ unidades. Lo que falta entre (costo + ganancia) y el techo son los costos fijos repartidos entre las unidades.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="3" t="inlineStr">
+        <is>
           <t>Cómo se lee</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="26" customHeight="1">
-      <c r="B18" s="4" t="inlineStr">
+    <row r="19" ht="28" customHeight="1">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Cantidad: cuántas acciones o personas hubo en ese paso con los supuestos del escenario en uso.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="26" customHeight="1">
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>% que pasa: de los que estaban en el paso anterior (o en el paso que indica la nota), cuántos llegan a este. % que se pierde es el complemento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="26" customHeight="1">
+    <row r="20" ht="28" customHeight="1">
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>% acumulado: cuántos llegan a este paso por cada 100 unidades que compra la pauta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="26" customHeight="1">
+          <t>% que pasa: de los que estaban en el paso anterior (o en el paso que indica la nota), cuántos llegan a este. % acumulado: cuántos llegan a este paso por cada 100 unidades que compra la pauta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
       <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Costo por paso: inversión ÷ cantidad. Es lo que te está costando hoy cada persona que llega a ese paso.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="26" customHeight="1">
+    <row r="22" ht="28" customHeight="1">
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Techo por paso: lo máximo que podrías pagar por ese paso sin perder plata, si lo demás se mantiene. Comparalo con el costo por paso: si el costo está por encima del techo, ese paso está caro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="26" customHeight="1">
+          <t>Ganancia por paso: ganancia del período ÷ cantidad. Lo que te queda por cada persona de ese paso después de pagar la pauta, las comisiones, los reembolsos y los fijos. La ganancia por visita es la métrica más valiosa del embudo: resume todo lo que pasa después.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Ganancia por paso: la ganancia del período dividida por la cantidad de ese paso. Es la otra cara del costo: cuánto te queda por cada visita, por cada lead, por cada comprador. La ganancia por visita es la métrica más valiosa del embudo: resume todo lo que pasa después.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="26" customHeight="1">
+          <t>Techo por paso: lo que cada persona de ese paso genera en cash neto (cash neto menos costos por unidad, dividido por la cantidad). Es lo máximo que podrías pagar por ese paso antes de que la ganancia llegue a cero, si lo demás se mantiene. Por eso siempre es mayor que la ganancia: techo = costo + ganancia + fijos repartidos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
       <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Los bumps, las OTOs y la ascensión no tienen costo propio: se pagan con el CPA del comprador principal y se miden por lo que suman al AOV.</t>
@@ -3354,14 +3324,13 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="B24:J24"/>
-    <mergeCell ref="B19:J19"/>
-    <mergeCell ref="B20:J20"/>
-    <mergeCell ref="B22:J22"/>
-    <mergeCell ref="B23:J23"/>
-    <mergeCell ref="B18:J18"/>
-    <mergeCell ref="B21:J21"/>
+  <mergeCells count="6">
+    <mergeCell ref="B21:I21"/>
+    <mergeCell ref="B24:I24"/>
+    <mergeCell ref="B20:I20"/>
+    <mergeCell ref="B22:I22"/>
+    <mergeCell ref="B19:I19"/>
+    <mergeCell ref="B23:I23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
@@ -3504,7 +3473,7 @@
           <t>Costo por visita a la página de ventas (VSL)</t>
         </is>
       </c>
-      <c r="C9" s="17">
+      <c r="C9" s="18">
         <f>IF('Supuestos'!$C$6=1,D9,IF('Supuestos'!$C$6=2,E9,F9))</f>
         <v/>
       </c>
@@ -3547,7 +3516,7 @@
           <t>% de visitas que llegan al checkout</t>
         </is>
       </c>
-      <c r="C12" s="18">
+      <c r="C12" s="17">
         <f>IF('Supuestos'!$C$6=1,D12,IF('Supuestos'!$C$6=2,E12,F12))</f>
         <v/>
       </c>
@@ -3577,7 +3546,7 @@
           <t>% de checkouts que terminan en compra</t>
         </is>
       </c>
-      <c r="C13" s="18">
+      <c r="C13" s="17">
         <f>IF('Supuestos'!$C$6=1,D13,IF('Supuestos'!$C$6=2,E13,F13))</f>
         <v/>
       </c>
@@ -3660,7 +3629,7 @@
           <t>Bump 1: % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C18" s="18">
+      <c r="C18" s="17">
         <f>IF('Supuestos'!$C$6=1,D18,IF('Supuestos'!$C$6=2,E18,F18))</f>
         <v/>
       </c>
@@ -3706,7 +3675,7 @@
           <t>Bump 2: % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C20" s="18">
+      <c r="C20" s="17">
         <f>IF('Supuestos'!$C$6=1,D20,IF('Supuestos'!$C$6=2,E20,F20))</f>
         <v/>
       </c>
@@ -3752,7 +3721,7 @@
           <t>OTO 1: % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C22" s="18">
+      <c r="C22" s="17">
         <f>IF('Supuestos'!$C$6=1,D22,IF('Supuestos'!$C$6=2,E22,F22))</f>
         <v/>
       </c>
@@ -3798,7 +3767,7 @@
           <t>OTO 2: % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C24" s="18">
+      <c r="C24" s="17">
         <f>IF('Supuestos'!$C$6=1,D24,IF('Supuestos'!$C$6=2,E24,F24))</f>
         <v/>
       </c>
@@ -3844,7 +3813,7 @@
           <t>OTO 3: % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C26" s="18">
+      <c r="C26" s="17">
         <f>IF('Supuestos'!$C$6=1,D26,IF('Supuestos'!$C$6=2,E26,F26))</f>
         <v/>
       </c>
@@ -3890,7 +3859,7 @@
           <t>OTO 4: % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C28" s="18">
+      <c r="C28" s="17">
         <f>IF('Supuestos'!$C$6=1,D28,IF('Supuestos'!$C$6=2,E28,F28))</f>
         <v/>
       </c>
@@ -3936,7 +3905,7 @@
           <t>Ascensión (programa de mayor valor): % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C30" s="18">
+      <c r="C30" s="17">
         <f>IF('Supuestos'!$C$6=1,D30,IF('Supuestos'!$C$6=2,E30,F30))</f>
         <v/>
       </c>
@@ -4329,7 +4298,7 @@
           <t>Costo por visita (unidad de adquisición)</t>
         </is>
       </c>
-      <c r="C7" s="17">
+      <c r="C7" s="18">
         <f>'Supuestos'!$C$9</f>
         <v/>
       </c>
@@ -4738,7 +4707,7 @@
           <t>Facturado por visita</t>
         </is>
       </c>
-      <c r="C33" s="17">
+      <c r="C33" s="18">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$29/'Modelo'!$C$8)</f>
         <v/>
       </c>
@@ -4907,7 +4876,7 @@
           <t>Margen sobre cash</t>
         </is>
       </c>
-      <c r="C44" s="18">
+      <c r="C44" s="17">
         <f>IF('Modelo'!$C$35=0,0,'Modelo'!$C$41/'Modelo'!$C$35)</f>
         <v/>
       </c>
@@ -4996,7 +4965,7 @@
           <t>Techo de costo por checkout</t>
         </is>
       </c>
-      <c r="C50" s="17">
+      <c r="C50" s="18">
         <f>IF('Supuestos'!$C$12=0,0,'Modelo'!$C$47/'Supuestos'!$C$12)</f>
         <v/>
       </c>
@@ -5028,7 +4997,7 @@
           <t>Objetivo de CPA</t>
         </is>
       </c>
-      <c r="C52" s="17">
+      <c r="C52" s="18">
         <f>'Modelo'!$C$51/(1+'Supuestos'!$C$46)</f>
         <v/>
       </c>
@@ -5044,7 +5013,7 @@
           <t>Cash neto por comprador (AOV neto)</t>
         </is>
       </c>
-      <c r="C53" s="17">
+      <c r="C53" s="18">
         <f>IF('Modelo'!$C$10=0,0,('Modelo'!$C$39-'Modelo'!$C$40)/'Modelo'!$C$10)</f>
         <v/>
       </c>
@@ -5158,7 +5127,7 @@
           <t>Ganancia por checkout</t>
         </is>
       </c>
-      <c r="C61" s="17">
+      <c r="C61" s="18">
         <f>IF('Modelo'!$C$9=0,0,'Modelo'!$C$41/'Modelo'!$C$9)</f>
         <v/>
       </c>
@@ -5906,23 +5875,23 @@
           <t>Costo máximo (facturado por unidad ÷ ROAS)</t>
         </is>
       </c>
-      <c r="C46" s="17">
+      <c r="C46" s="18">
         <f>IF(C45=0,0,'Modelo'!$C$33/C45)</f>
         <v/>
       </c>
-      <c r="D46" s="17">
+      <c r="D46" s="18">
         <f>IF(D45=0,0,'Modelo'!$C$33/D45)</f>
         <v/>
       </c>
-      <c r="E46" s="17">
+      <c r="E46" s="18">
         <f>IF(E45=0,0,'Modelo'!$C$33/E45)</f>
         <v/>
       </c>
-      <c r="F46" s="17">
+      <c r="F46" s="18">
         <f>IF(F45=0,0,'Modelo'!$C$33/F45)</f>
         <v/>
       </c>
-      <c r="G46" s="17">
+      <c r="G46" s="18">
         <f>IF(G45=0,0,'Modelo'!$C$33/G45)</f>
         <v/>
       </c>
@@ -6196,7 +6165,7 @@
         <f>D7-$D$6</f>
         <v/>
       </c>
-      <c r="F7" s="18">
+      <c r="F7" s="17">
         <f>IF($D$6=0,0,E7/ABS($D$6))</f>
         <v/>
       </c>
@@ -6224,7 +6193,7 @@
         <f>D8-$D$6</f>
         <v/>
       </c>
-      <c r="F8" s="18">
+      <c r="F8" s="17">
         <f>IF($D$6=0,0,E8/ABS($D$6))</f>
         <v/>
       </c>
@@ -6252,7 +6221,7 @@
         <f>D9-$D$6</f>
         <v/>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="17">
         <f>IF($D$6=0,0,E9/ABS($D$6))</f>
         <v/>
       </c>
@@ -6280,7 +6249,7 @@
         <f>D10-$D$6</f>
         <v/>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="17">
         <f>IF($D$6=0,0,E10/ABS($D$6))</f>
         <v/>
       </c>
@@ -6308,7 +6277,7 @@
         <f>D11-$D$6</f>
         <v/>
       </c>
-      <c r="F11" s="18">
+      <c r="F11" s="17">
         <f>IF($D$6=0,0,E11/ABS($D$6))</f>
         <v/>
       </c>
@@ -6336,7 +6305,7 @@
         <f>D12-$D$6</f>
         <v/>
       </c>
-      <c r="F12" s="18">
+      <c r="F12" s="17">
         <f>IF($D$6=0,0,E12/ABS($D$6))</f>
         <v/>
       </c>
@@ -6364,7 +6333,7 @@
         <f>D13-$D$6</f>
         <v/>
       </c>
-      <c r="F13" s="18">
+      <c r="F13" s="17">
         <f>IF($D$6=0,0,E13/ABS($D$6))</f>
         <v/>
       </c>
@@ -6392,7 +6361,7 @@
         <f>D14-$D$6</f>
         <v/>
       </c>
-      <c r="F14" s="18">
+      <c r="F14" s="17">
         <f>IF($D$6=0,0,E14/ABS($D$6))</f>
         <v/>
       </c>
@@ -7774,15 +7743,15 @@
         <f>IF(COUNT(N7:N15)&lt;9,"",IF(N8=0,0,N7/N8))</f>
         <v/>
       </c>
-      <c r="O17" s="17">
+      <c r="O17" s="18">
         <f>IF(COUNT(C17:N17)=0,"",AVERAGE(C17:N17))</f>
         <v/>
       </c>
-      <c r="P17" s="17">
+      <c r="P17" s="18">
         <f>IF(COUNT(C17:N17)=0,"",MAX(C17:N17))</f>
         <v/>
       </c>
-      <c r="Q17" s="17">
+      <c r="Q17" s="18">
         <f>IF(COUNT(C17:N17)=0,"",MIN(C17:N17))</f>
         <v/>
       </c>
@@ -7793,63 +7762,63 @@
           <t>% visitas → checkout</t>
         </is>
       </c>
-      <c r="C18" s="18">
+      <c r="C18" s="17">
         <f>IF(COUNT(C7:C15)&lt;9,"",IF(C8=0,0,C9/C8))</f>
         <v/>
       </c>
-      <c r="D18" s="18">
+      <c r="D18" s="17">
         <f>IF(COUNT(D7:D15)&lt;9,"",IF(D8=0,0,D9/D8))</f>
         <v/>
       </c>
-      <c r="E18" s="18">
+      <c r="E18" s="17">
         <f>IF(COUNT(E7:E15)&lt;9,"",IF(E8=0,0,E9/E8))</f>
         <v/>
       </c>
-      <c r="F18" s="18">
+      <c r="F18" s="17">
         <f>IF(COUNT(F7:F15)&lt;9,"",IF(F8=0,0,F9/F8))</f>
         <v/>
       </c>
-      <c r="G18" s="18">
+      <c r="G18" s="17">
         <f>IF(COUNT(G7:G15)&lt;9,"",IF(G8=0,0,G9/G8))</f>
         <v/>
       </c>
-      <c r="H18" s="18">
+      <c r="H18" s="17">
         <f>IF(COUNT(H7:H15)&lt;9,"",IF(H8=0,0,H9/H8))</f>
         <v/>
       </c>
-      <c r="I18" s="18">
+      <c r="I18" s="17">
         <f>IF(COUNT(I7:I15)&lt;9,"",IF(I8=0,0,I9/I8))</f>
         <v/>
       </c>
-      <c r="J18" s="18">
+      <c r="J18" s="17">
         <f>IF(COUNT(J7:J15)&lt;9,"",IF(J8=0,0,J9/J8))</f>
         <v/>
       </c>
-      <c r="K18" s="18">
+      <c r="K18" s="17">
         <f>IF(COUNT(K7:K15)&lt;9,"",IF(K8=0,0,K9/K8))</f>
         <v/>
       </c>
-      <c r="L18" s="18">
+      <c r="L18" s="17">
         <f>IF(COUNT(L7:L15)&lt;9,"",IF(L8=0,0,L9/L8))</f>
         <v/>
       </c>
-      <c r="M18" s="18">
+      <c r="M18" s="17">
         <f>IF(COUNT(M7:M15)&lt;9,"",IF(M8=0,0,M9/M8))</f>
         <v/>
       </c>
-      <c r="N18" s="18">
+      <c r="N18" s="17">
         <f>IF(COUNT(N7:N15)&lt;9,"",IF(N8=0,0,N9/N8))</f>
         <v/>
       </c>
-      <c r="O18" s="18">
+      <c r="O18" s="17">
         <f>IF(COUNT(C18:N18)=0,"",AVERAGE(C18:N18))</f>
         <v/>
       </c>
-      <c r="P18" s="18">
+      <c r="P18" s="17">
         <f>IF(COUNT(C18:N18)=0,"",MAX(C18:N18))</f>
         <v/>
       </c>
-      <c r="Q18" s="18">
+      <c r="Q18" s="17">
         <f>IF(COUNT(C18:N18)=0,"",MIN(C18:N18))</f>
         <v/>
       </c>
@@ -7860,63 +7829,63 @@
           <t>% checkout → compra</t>
         </is>
       </c>
-      <c r="C19" s="18">
+      <c r="C19" s="17">
         <f>IF(COUNT(C7:C15)&lt;9,"",IF(C9=0,0,C10/C9))</f>
         <v/>
       </c>
-      <c r="D19" s="18">
+      <c r="D19" s="17">
         <f>IF(COUNT(D7:D15)&lt;9,"",IF(D9=0,0,D10/D9))</f>
         <v/>
       </c>
-      <c r="E19" s="18">
+      <c r="E19" s="17">
         <f>IF(COUNT(E7:E15)&lt;9,"",IF(E9=0,0,E10/E9))</f>
         <v/>
       </c>
-      <c r="F19" s="18">
+      <c r="F19" s="17">
         <f>IF(COUNT(F7:F15)&lt;9,"",IF(F9=0,0,F10/F9))</f>
         <v/>
       </c>
-      <c r="G19" s="18">
+      <c r="G19" s="17">
         <f>IF(COUNT(G7:G15)&lt;9,"",IF(G9=0,0,G10/G9))</f>
         <v/>
       </c>
-      <c r="H19" s="18">
+      <c r="H19" s="17">
         <f>IF(COUNT(H7:H15)&lt;9,"",IF(H9=0,0,H10/H9))</f>
         <v/>
       </c>
-      <c r="I19" s="18">
+      <c r="I19" s="17">
         <f>IF(COUNT(I7:I15)&lt;9,"",IF(I9=0,0,I10/I9))</f>
         <v/>
       </c>
-      <c r="J19" s="18">
+      <c r="J19" s="17">
         <f>IF(COUNT(J7:J15)&lt;9,"",IF(J9=0,0,J10/J9))</f>
         <v/>
       </c>
-      <c r="K19" s="18">
+      <c r="K19" s="17">
         <f>IF(COUNT(K7:K15)&lt;9,"",IF(K9=0,0,K10/K9))</f>
         <v/>
       </c>
-      <c r="L19" s="18">
+      <c r="L19" s="17">
         <f>IF(COUNT(L7:L15)&lt;9,"",IF(L9=0,0,L10/L9))</f>
         <v/>
       </c>
-      <c r="M19" s="18">
+      <c r="M19" s="17">
         <f>IF(COUNT(M7:M15)&lt;9,"",IF(M9=0,0,M10/M9))</f>
         <v/>
       </c>
-      <c r="N19" s="18">
+      <c r="N19" s="17">
         <f>IF(COUNT(N7:N15)&lt;9,"",IF(N9=0,0,N10/N9))</f>
         <v/>
       </c>
-      <c r="O19" s="18">
+      <c r="O19" s="17">
         <f>IF(COUNT(C19:N19)=0,"",AVERAGE(C19:N19))</f>
         <v/>
       </c>
-      <c r="P19" s="18">
+      <c r="P19" s="17">
         <f>IF(COUNT(C19:N19)=0,"",MAX(C19:N19))</f>
         <v/>
       </c>
-      <c r="Q19" s="18">
+      <c r="Q19" s="17">
         <f>IF(COUNT(C19:N19)=0,"",MIN(C19:N19))</f>
         <v/>
       </c>
@@ -7927,63 +7896,63 @@
           <t>CPA real</t>
         </is>
       </c>
-      <c r="C20" s="17">
+      <c r="C20" s="18">
         <f>IF(COUNT(C7:C15)&lt;9,"",IF(C10=0,0,C7/C10))</f>
         <v/>
       </c>
-      <c r="D20" s="17">
+      <c r="D20" s="18">
         <f>IF(COUNT(D7:D15)&lt;9,"",IF(D10=0,0,D7/D10))</f>
         <v/>
       </c>
-      <c r="E20" s="17">
+      <c r="E20" s="18">
         <f>IF(COUNT(E7:E15)&lt;9,"",IF(E10=0,0,E7/E10))</f>
         <v/>
       </c>
-      <c r="F20" s="17">
+      <c r="F20" s="18">
         <f>IF(COUNT(F7:F15)&lt;9,"",IF(F10=0,0,F7/F10))</f>
         <v/>
       </c>
-      <c r="G20" s="17">
+      <c r="G20" s="18">
         <f>IF(COUNT(G7:G15)&lt;9,"",IF(G10=0,0,G7/G10))</f>
         <v/>
       </c>
-      <c r="H20" s="17">
+      <c r="H20" s="18">
         <f>IF(COUNT(H7:H15)&lt;9,"",IF(H10=0,0,H7/H10))</f>
         <v/>
       </c>
-      <c r="I20" s="17">
+      <c r="I20" s="18">
         <f>IF(COUNT(I7:I15)&lt;9,"",IF(I10=0,0,I7/I10))</f>
         <v/>
       </c>
-      <c r="J20" s="17">
+      <c r="J20" s="18">
         <f>IF(COUNT(J7:J15)&lt;9,"",IF(J10=0,0,J7/J10))</f>
         <v/>
       </c>
-      <c r="K20" s="17">
+      <c r="K20" s="18">
         <f>IF(COUNT(K7:K15)&lt;9,"",IF(K10=0,0,K7/K10))</f>
         <v/>
       </c>
-      <c r="L20" s="17">
+      <c r="L20" s="18">
         <f>IF(COUNT(L7:L15)&lt;9,"",IF(L10=0,0,L7/L10))</f>
         <v/>
       </c>
-      <c r="M20" s="17">
+      <c r="M20" s="18">
         <f>IF(COUNT(M7:M15)&lt;9,"",IF(M10=0,0,M7/M10))</f>
         <v/>
       </c>
-      <c r="N20" s="17">
+      <c r="N20" s="18">
         <f>IF(COUNT(N7:N15)&lt;9,"",IF(N10=0,0,N7/N10))</f>
         <v/>
       </c>
-      <c r="O20" s="17">
+      <c r="O20" s="18">
         <f>IF(COUNT(C20:N20)=0,"",AVERAGE(C20:N20))</f>
         <v/>
       </c>
-      <c r="P20" s="17">
+      <c r="P20" s="18">
         <f>IF(COUNT(C20:N20)=0,"",MAX(C20:N20))</f>
         <v/>
       </c>
-      <c r="Q20" s="17">
+      <c r="Q20" s="18">
         <f>IF(COUNT(C20:N20)=0,"",MIN(C20:N20))</f>
         <v/>
       </c>
@@ -7994,63 +7963,63 @@
           <t>Cash por comprador</t>
         </is>
       </c>
-      <c r="C21" s="17">
+      <c r="C21" s="18">
         <f>IF(COUNT(C7:C15)&lt;9,"",IF(C10=0,0,C15/C10))</f>
         <v/>
       </c>
-      <c r="D21" s="17">
+      <c r="D21" s="18">
         <f>IF(COUNT(D7:D15)&lt;9,"",IF(D10=0,0,D15/D10))</f>
         <v/>
       </c>
-      <c r="E21" s="17">
+      <c r="E21" s="18">
         <f>IF(COUNT(E7:E15)&lt;9,"",IF(E10=0,0,E15/E10))</f>
         <v/>
       </c>
-      <c r="F21" s="17">
+      <c r="F21" s="18">
         <f>IF(COUNT(F7:F15)&lt;9,"",IF(F10=0,0,F15/F10))</f>
         <v/>
       </c>
-      <c r="G21" s="17">
+      <c r="G21" s="18">
         <f>IF(COUNT(G7:G15)&lt;9,"",IF(G10=0,0,G15/G10))</f>
         <v/>
       </c>
-      <c r="H21" s="17">
+      <c r="H21" s="18">
         <f>IF(COUNT(H7:H15)&lt;9,"",IF(H10=0,0,H15/H10))</f>
         <v/>
       </c>
-      <c r="I21" s="17">
+      <c r="I21" s="18">
         <f>IF(COUNT(I7:I15)&lt;9,"",IF(I10=0,0,I15/I10))</f>
         <v/>
       </c>
-      <c r="J21" s="17">
+      <c r="J21" s="18">
         <f>IF(COUNT(J7:J15)&lt;9,"",IF(J10=0,0,J15/J10))</f>
         <v/>
       </c>
-      <c r="K21" s="17">
+      <c r="K21" s="18">
         <f>IF(COUNT(K7:K15)&lt;9,"",IF(K10=0,0,K15/K10))</f>
         <v/>
       </c>
-      <c r="L21" s="17">
+      <c r="L21" s="18">
         <f>IF(COUNT(L7:L15)&lt;9,"",IF(L10=0,0,L15/L10))</f>
         <v/>
       </c>
-      <c r="M21" s="17">
+      <c r="M21" s="18">
         <f>IF(COUNT(M7:M15)&lt;9,"",IF(M10=0,0,M15/M10))</f>
         <v/>
       </c>
-      <c r="N21" s="17">
+      <c r="N21" s="18">
         <f>IF(COUNT(N7:N15)&lt;9,"",IF(N10=0,0,N15/N10))</f>
         <v/>
       </c>
-      <c r="O21" s="17">
+      <c r="O21" s="18">
         <f>IF(COUNT(C21:N21)=0,"",AVERAGE(C21:N21))</f>
         <v/>
       </c>
-      <c r="P21" s="17">
+      <c r="P21" s="18">
         <f>IF(COUNT(C21:N21)=0,"",MAX(C21:N21))</f>
         <v/>
       </c>
-      <c r="Q21" s="17">
+      <c r="Q21" s="18">
         <f>IF(COUNT(C21:N21)=0,"",MIN(C21:N21))</f>
         <v/>
       </c>
@@ -8109,15 +8078,15 @@
         <f>IF(COUNT(N7:N15)&lt;9,"",IF(N8=0,0,(N14*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)-N8*'Supuestos'!$C$36)/N8))</f>
         <v/>
       </c>
-      <c r="O22" s="17">
+      <c r="O22" s="18">
         <f>IF(COUNT(C22:N22)=0,"",AVERAGE(C22:N22))</f>
         <v/>
       </c>
-      <c r="P22" s="17">
+      <c r="P22" s="18">
         <f>IF(COUNT(C22:N22)=0,"",MAX(C22:N22))</f>
         <v/>
       </c>
-      <c r="Q22" s="17">
+      <c r="Q22" s="18">
         <f>IF(COUNT(C22:N22)=0,"",MIN(C22:N22))</f>
         <v/>
       </c>
@@ -8310,15 +8279,15 @@
         <f>IF(COUNT(N7:N15)&lt;9,"",IF(N8=0,0,(N14*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)-N8*'Supuestos'!$C$36-'Supuestos'!$C$37-N7)/N8))</f>
         <v/>
       </c>
-      <c r="O25" s="17">
+      <c r="O25" s="18">
         <f>IF(COUNT(C25:N25)=0,"",AVERAGE(C25:N25))</f>
         <v/>
       </c>
-      <c r="P25" s="17">
+      <c r="P25" s="18">
         <f>IF(COUNT(C25:N25)=0,"",MAX(C25:N25))</f>
         <v/>
       </c>
-      <c r="Q25" s="17">
+      <c r="Q25" s="18">
         <f>IF(COUNT(C25:N25)=0,"",MIN(C25:N25))</f>
         <v/>
       </c>
@@ -8463,63 +8432,63 @@
           <t>Techo móvil (mediana de tus últimas 4 columnas; al inicio, el del modelo)</t>
         </is>
       </c>
-      <c r="C28" s="17">
+      <c r="C28" s="18">
         <f>IF(COUNT(C7:C15)&lt;9,"",'Modelo'!$C$48)</f>
         <v/>
       </c>
-      <c r="D28" s="17">
+      <c r="D28" s="18">
         <f>IF(COUNT(D7:D15)&lt;9,"",IF(COUNT(C22:C22)&gt;0,MEDIAN(C22:C22),'Modelo'!$C$48))</f>
         <v/>
       </c>
-      <c r="E28" s="17">
+      <c r="E28" s="18">
         <f>IF(COUNT(E7:E15)&lt;9,"",IF(COUNT(C22:D22)&gt;0,MEDIAN(C22:D22),'Modelo'!$C$48))</f>
         <v/>
       </c>
-      <c r="F28" s="17">
+      <c r="F28" s="18">
         <f>IF(COUNT(F7:F15)&lt;9,"",IF(COUNT(C22:E22)&gt;0,MEDIAN(C22:E22),'Modelo'!$C$48))</f>
         <v/>
       </c>
-      <c r="G28" s="17">
+      <c r="G28" s="18">
         <f>IF(COUNT(G7:G15)&lt;9,"",IF(COUNT(C22:F22)&gt;0,MEDIAN(C22:F22),'Modelo'!$C$48))</f>
         <v/>
       </c>
-      <c r="H28" s="17">
+      <c r="H28" s="18">
         <f>IF(COUNT(H7:H15)&lt;9,"",IF(COUNT(D22:G22)&gt;0,MEDIAN(D22:G22),'Modelo'!$C$48))</f>
         <v/>
       </c>
-      <c r="I28" s="17">
+      <c r="I28" s="18">
         <f>IF(COUNT(I7:I15)&lt;9,"",IF(COUNT(E22:H22)&gt;0,MEDIAN(E22:H22),'Modelo'!$C$48))</f>
         <v/>
       </c>
-      <c r="J28" s="17">
+      <c r="J28" s="18">
         <f>IF(COUNT(J7:J15)&lt;9,"",IF(COUNT(F22:I22)&gt;0,MEDIAN(F22:I22),'Modelo'!$C$48))</f>
         <v/>
       </c>
-      <c r="K28" s="17">
+      <c r="K28" s="18">
         <f>IF(COUNT(K7:K15)&lt;9,"",IF(COUNT(G22:J22)&gt;0,MEDIAN(G22:J22),'Modelo'!$C$48))</f>
         <v/>
       </c>
-      <c r="L28" s="17">
+      <c r="L28" s="18">
         <f>IF(COUNT(L7:L15)&lt;9,"",IF(COUNT(H22:K22)&gt;0,MEDIAN(H22:K22),'Modelo'!$C$48))</f>
         <v/>
       </c>
-      <c r="M28" s="17">
+      <c r="M28" s="18">
         <f>IF(COUNT(M7:M15)&lt;9,"",IF(COUNT(I22:L22)&gt;0,MEDIAN(I22:L22),'Modelo'!$C$48))</f>
         <v/>
       </c>
-      <c r="N28" s="17">
+      <c r="N28" s="18">
         <f>IF(COUNT(N7:N15)&lt;9,"",IF(COUNT(J22:M22)&gt;0,MEDIAN(J22:M22),'Modelo'!$C$48))</f>
         <v/>
       </c>
-      <c r="O28" s="17">
+      <c r="O28" s="18">
         <f>IF(COUNT(C28:N28)=0,"",AVERAGE(C28:N28))</f>
         <v/>
       </c>
-      <c r="P28" s="17">
+      <c r="P28" s="18">
         <f>IF(COUNT(C28:N28)=0,"",MAX(C28:N28))</f>
         <v/>
       </c>
-      <c r="Q28" s="17">
+      <c r="Q28" s="18">
         <f>IF(COUNT(C28:N28)=0,"",MIN(C28:N28))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Skill v3 plug and play: README de comportamiento, perfil de la persona (perfil/mi_embudo.json + PERFIL.md), proyección a 12 meses con caja necesaria y umbrales al frente; Simulador: validación, columna Rango y chequeos con los números del Simulador
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/01_Modelo_Financiero_Embudo_Low_Ticket_Bumps_Upsells.xlsx
+++ b/excel/01_Modelo_Financiero_Embudo_Low_Ticket_Bumps_Upsells.xlsx
@@ -179,6 +179,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -197,7 +198,6 @@
     <xf numFmtId="167" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1050,33 +1050,33 @@
           <t>Inversión en publicidad</t>
         </is>
       </c>
-      <c r="C7" s="18" t="n">
+      <c r="C7" s="19" t="n">
         <v>9000</v>
       </c>
-      <c r="D7" s="18" t="n">
+      <c r="D7" s="19" t="n">
         <v>9500</v>
       </c>
-      <c r="E7" s="18" t="n">
+      <c r="E7" s="19" t="n">
         <v>10500</v>
       </c>
-      <c r="F7" s="18" t="n"/>
-      <c r="G7" s="18" t="n"/>
-      <c r="H7" s="18" t="n"/>
-      <c r="I7" s="18" t="n"/>
-      <c r="J7" s="18" t="n"/>
-      <c r="K7" s="18" t="n"/>
-      <c r="L7" s="18" t="n"/>
-      <c r="M7" s="18" t="n"/>
-      <c r="N7" s="18" t="n"/>
-      <c r="O7" s="19">
+      <c r="F7" s="19" t="n"/>
+      <c r="G7" s="19" t="n"/>
+      <c r="H7" s="19" t="n"/>
+      <c r="I7" s="19" t="n"/>
+      <c r="J7" s="19" t="n"/>
+      <c r="K7" s="19" t="n"/>
+      <c r="L7" s="19" t="n"/>
+      <c r="M7" s="19" t="n"/>
+      <c r="N7" s="19" t="n"/>
+      <c r="O7" s="20">
         <f>IF(COUNT(C7:N7)=0,"",AVERAGE(C7:N7))</f>
         <v/>
       </c>
-      <c r="P7" s="19">
+      <c r="P7" s="20">
         <f>IF(COUNT(C7:N7)=0,"",MAX(C7:N7))</f>
         <v/>
       </c>
-      <c r="Q7" s="19">
+      <c r="Q7" s="20">
         <f>IF(COUNT(C7:N7)=0,"",MIN(C7:N7))</f>
         <v/>
       </c>
@@ -1087,33 +1087,33 @@
           <t>Visitas a la página</t>
         </is>
       </c>
-      <c r="C8" s="29" t="n">
+      <c r="C8" s="30" t="n">
         <v>30000</v>
       </c>
-      <c r="D8" s="29" t="n">
+      <c r="D8" s="30" t="n">
         <v>30200</v>
       </c>
-      <c r="E8" s="29" t="n">
+      <c r="E8" s="30" t="n">
         <v>29000</v>
       </c>
-      <c r="F8" s="29" t="n"/>
-      <c r="G8" s="29" t="n"/>
-      <c r="H8" s="29" t="n"/>
-      <c r="I8" s="29" t="n"/>
-      <c r="J8" s="29" t="n"/>
-      <c r="K8" s="29" t="n"/>
-      <c r="L8" s="29" t="n"/>
-      <c r="M8" s="29" t="n"/>
-      <c r="N8" s="29" t="n"/>
-      <c r="O8" s="21">
+      <c r="F8" s="30" t="n"/>
+      <c r="G8" s="30" t="n"/>
+      <c r="H8" s="30" t="n"/>
+      <c r="I8" s="30" t="n"/>
+      <c r="J8" s="30" t="n"/>
+      <c r="K8" s="30" t="n"/>
+      <c r="L8" s="30" t="n"/>
+      <c r="M8" s="30" t="n"/>
+      <c r="N8" s="30" t="n"/>
+      <c r="O8" s="22">
         <f>IF(COUNT(C8:N8)=0,"",AVERAGE(C8:N8))</f>
         <v/>
       </c>
-      <c r="P8" s="21">
+      <c r="P8" s="22">
         <f>IF(COUNT(C8:N8)=0,"",MAX(C8:N8))</f>
         <v/>
       </c>
-      <c r="Q8" s="21">
+      <c r="Q8" s="22">
         <f>IF(COUNT(C8:N8)=0,"",MIN(C8:N8))</f>
         <v/>
       </c>
@@ -1124,33 +1124,33 @@
           <t>Checkouts iniciados</t>
         </is>
       </c>
-      <c r="C9" s="29" t="n">
+      <c r="C9" s="30" t="n">
         <v>1050</v>
       </c>
-      <c r="D9" s="29" t="n">
+      <c r="D9" s="30" t="n">
         <v>1030</v>
       </c>
-      <c r="E9" s="29" t="n">
+      <c r="E9" s="30" t="n">
         <v>980</v>
       </c>
-      <c r="F9" s="29" t="n"/>
-      <c r="G9" s="29" t="n"/>
-      <c r="H9" s="29" t="n"/>
-      <c r="I9" s="29" t="n"/>
-      <c r="J9" s="29" t="n"/>
-      <c r="K9" s="29" t="n"/>
-      <c r="L9" s="29" t="n"/>
-      <c r="M9" s="29" t="n"/>
-      <c r="N9" s="29" t="n"/>
-      <c r="O9" s="21">
+      <c r="F9" s="30" t="n"/>
+      <c r="G9" s="30" t="n"/>
+      <c r="H9" s="30" t="n"/>
+      <c r="I9" s="30" t="n"/>
+      <c r="J9" s="30" t="n"/>
+      <c r="K9" s="30" t="n"/>
+      <c r="L9" s="30" t="n"/>
+      <c r="M9" s="30" t="n"/>
+      <c r="N9" s="30" t="n"/>
+      <c r="O9" s="22">
         <f>IF(COUNT(C9:N9)=0,"",AVERAGE(C9:N9))</f>
         <v/>
       </c>
-      <c r="P9" s="21">
+      <c r="P9" s="22">
         <f>IF(COUNT(C9:N9)=0,"",MAX(C9:N9))</f>
         <v/>
       </c>
-      <c r="Q9" s="21">
+      <c r="Q9" s="22">
         <f>IF(COUNT(C9:N9)=0,"",MIN(C9:N9))</f>
         <v/>
       </c>
@@ -1161,33 +1161,33 @@
           <t>Ventas del producto principal</t>
         </is>
       </c>
-      <c r="C10" s="29" t="n">
+      <c r="C10" s="30" t="n">
         <v>273</v>
       </c>
-      <c r="D10" s="29" t="n">
+      <c r="D10" s="30" t="n">
         <v>262</v>
       </c>
-      <c r="E10" s="29" t="n">
+      <c r="E10" s="30" t="n">
         <v>240</v>
       </c>
-      <c r="F10" s="29" t="n"/>
-      <c r="G10" s="29" t="n"/>
-      <c r="H10" s="29" t="n"/>
-      <c r="I10" s="29" t="n"/>
-      <c r="J10" s="29" t="n"/>
-      <c r="K10" s="29" t="n"/>
-      <c r="L10" s="29" t="n"/>
-      <c r="M10" s="29" t="n"/>
-      <c r="N10" s="29" t="n"/>
-      <c r="O10" s="21">
+      <c r="F10" s="30" t="n"/>
+      <c r="G10" s="30" t="n"/>
+      <c r="H10" s="30" t="n"/>
+      <c r="I10" s="30" t="n"/>
+      <c r="J10" s="30" t="n"/>
+      <c r="K10" s="30" t="n"/>
+      <c r="L10" s="30" t="n"/>
+      <c r="M10" s="30" t="n"/>
+      <c r="N10" s="30" t="n"/>
+      <c r="O10" s="22">
         <f>IF(COUNT(C10:N10)=0,"",AVERAGE(C10:N10))</f>
         <v/>
       </c>
-      <c r="P10" s="21">
+      <c r="P10" s="22">
         <f>IF(COUNT(C10:N10)=0,"",MAX(C10:N10))</f>
         <v/>
       </c>
-      <c r="Q10" s="21">
+      <c r="Q10" s="22">
         <f>IF(COUNT(C10:N10)=0,"",MIN(C10:N10))</f>
         <v/>
       </c>
@@ -1198,33 +1198,33 @@
           <t>Ventas de bumps (1 + 2)</t>
         </is>
       </c>
-      <c r="C11" s="29" t="n">
+      <c r="C11" s="30" t="n">
         <v>117</v>
       </c>
-      <c r="D11" s="29" t="n">
+      <c r="D11" s="30" t="n">
         <v>110</v>
       </c>
-      <c r="E11" s="29" t="n">
+      <c r="E11" s="30" t="n">
         <v>95</v>
       </c>
-      <c r="F11" s="29" t="n"/>
-      <c r="G11" s="29" t="n"/>
-      <c r="H11" s="29" t="n"/>
-      <c r="I11" s="29" t="n"/>
-      <c r="J11" s="29" t="n"/>
-      <c r="K11" s="29" t="n"/>
-      <c r="L11" s="29" t="n"/>
-      <c r="M11" s="29" t="n"/>
-      <c r="N11" s="29" t="n"/>
-      <c r="O11" s="21">
+      <c r="F11" s="30" t="n"/>
+      <c r="G11" s="30" t="n"/>
+      <c r="H11" s="30" t="n"/>
+      <c r="I11" s="30" t="n"/>
+      <c r="J11" s="30" t="n"/>
+      <c r="K11" s="30" t="n"/>
+      <c r="L11" s="30" t="n"/>
+      <c r="M11" s="30" t="n"/>
+      <c r="N11" s="30" t="n"/>
+      <c r="O11" s="22">
         <f>IF(COUNT(C11:N11)=0,"",AVERAGE(C11:N11))</f>
         <v/>
       </c>
-      <c r="P11" s="21">
+      <c r="P11" s="22">
         <f>IF(COUNT(C11:N11)=0,"",MAX(C11:N11))</f>
         <v/>
       </c>
-      <c r="Q11" s="21">
+      <c r="Q11" s="22">
         <f>IF(COUNT(C11:N11)=0,"",MIN(C11:N11))</f>
         <v/>
       </c>
@@ -1235,33 +1235,33 @@
           <t>Ventas de OTOs (1 a 4)</t>
         </is>
       </c>
-      <c r="C12" s="29" t="n">
+      <c r="C12" s="30" t="n">
         <v>63</v>
       </c>
-      <c r="D12" s="29" t="n">
+      <c r="D12" s="30" t="n">
         <v>58</v>
       </c>
-      <c r="E12" s="29" t="n">
+      <c r="E12" s="30" t="n">
         <v>52</v>
       </c>
-      <c r="F12" s="29" t="n"/>
-      <c r="G12" s="29" t="n"/>
-      <c r="H12" s="29" t="n"/>
-      <c r="I12" s="29" t="n"/>
-      <c r="J12" s="29" t="n"/>
-      <c r="K12" s="29" t="n"/>
-      <c r="L12" s="29" t="n"/>
-      <c r="M12" s="29" t="n"/>
-      <c r="N12" s="29" t="n"/>
-      <c r="O12" s="21">
+      <c r="F12" s="30" t="n"/>
+      <c r="G12" s="30" t="n"/>
+      <c r="H12" s="30" t="n"/>
+      <c r="I12" s="30" t="n"/>
+      <c r="J12" s="30" t="n"/>
+      <c r="K12" s="30" t="n"/>
+      <c r="L12" s="30" t="n"/>
+      <c r="M12" s="30" t="n"/>
+      <c r="N12" s="30" t="n"/>
+      <c r="O12" s="22">
         <f>IF(COUNT(C12:N12)=0,"",AVERAGE(C12:N12))</f>
         <v/>
       </c>
-      <c r="P12" s="21">
+      <c r="P12" s="22">
         <f>IF(COUNT(C12:N12)=0,"",MAX(C12:N12))</f>
         <v/>
       </c>
-      <c r="Q12" s="21">
+      <c r="Q12" s="22">
         <f>IF(COUNT(C12:N12)=0,"",MIN(C12:N12))</f>
         <v/>
       </c>
@@ -1272,33 +1272,33 @@
           <t>Ventas de la ascensión (programa)</t>
         </is>
       </c>
-      <c r="C13" s="29" t="n">
+      <c r="C13" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="D13" s="29" t="n">
+      <c r="D13" s="30" t="n">
         <v>6</v>
       </c>
-      <c r="E13" s="29" t="n">
+      <c r="E13" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="F13" s="29" t="n"/>
-      <c r="G13" s="29" t="n"/>
-      <c r="H13" s="29" t="n"/>
-      <c r="I13" s="29" t="n"/>
-      <c r="J13" s="29" t="n"/>
-      <c r="K13" s="29" t="n"/>
-      <c r="L13" s="29" t="n"/>
-      <c r="M13" s="29" t="n"/>
-      <c r="N13" s="29" t="n"/>
-      <c r="O13" s="21">
+      <c r="F13" s="30" t="n"/>
+      <c r="G13" s="30" t="n"/>
+      <c r="H13" s="30" t="n"/>
+      <c r="I13" s="30" t="n"/>
+      <c r="J13" s="30" t="n"/>
+      <c r="K13" s="30" t="n"/>
+      <c r="L13" s="30" t="n"/>
+      <c r="M13" s="30" t="n"/>
+      <c r="N13" s="30" t="n"/>
+      <c r="O13" s="22">
         <f>IF(COUNT(C13:N13)=0,"",AVERAGE(C13:N13))</f>
         <v/>
       </c>
-      <c r="P13" s="21">
+      <c r="P13" s="22">
         <f>IF(COUNT(C13:N13)=0,"",MAX(C13:N13))</f>
         <v/>
       </c>
-      <c r="Q13" s="21">
+      <c r="Q13" s="22">
         <f>IF(COUNT(C13:N13)=0,"",MIN(C13:N13))</f>
         <v/>
       </c>
@@ -1309,33 +1309,33 @@
           <t>Facturado del mes (a precio de lista)</t>
         </is>
       </c>
-      <c r="C14" s="18" t="n">
+      <c r="C14" s="19" t="n">
         <v>15900</v>
       </c>
-      <c r="D14" s="18" t="n">
+      <c r="D14" s="19" t="n">
         <v>15400</v>
       </c>
-      <c r="E14" s="18" t="n">
+      <c r="E14" s="19" t="n">
         <v>13700</v>
       </c>
-      <c r="F14" s="18" t="n"/>
-      <c r="G14" s="18" t="n"/>
-      <c r="H14" s="18" t="n"/>
-      <c r="I14" s="18" t="n"/>
-      <c r="J14" s="18" t="n"/>
-      <c r="K14" s="18" t="n"/>
-      <c r="L14" s="18" t="n"/>
-      <c r="M14" s="18" t="n"/>
-      <c r="N14" s="18" t="n"/>
-      <c r="O14" s="19">
+      <c r="F14" s="19" t="n"/>
+      <c r="G14" s="19" t="n"/>
+      <c r="H14" s="19" t="n"/>
+      <c r="I14" s="19" t="n"/>
+      <c r="J14" s="19" t="n"/>
+      <c r="K14" s="19" t="n"/>
+      <c r="L14" s="19" t="n"/>
+      <c r="M14" s="19" t="n"/>
+      <c r="N14" s="19" t="n"/>
+      <c r="O14" s="20">
         <f>IF(COUNT(C14:N14)=0,"",AVERAGE(C14:N14))</f>
         <v/>
       </c>
-      <c r="P14" s="19">
+      <c r="P14" s="20">
         <f>IF(COUNT(C14:N14)=0,"",MAX(C14:N14))</f>
         <v/>
       </c>
-      <c r="Q14" s="19">
+      <c r="Q14" s="20">
         <f>IF(COUNT(C14:N14)=0,"",MIN(C14:N14))</f>
         <v/>
       </c>
@@ -1346,33 +1346,33 @@
           <t>Cash cobrado en el mes</t>
         </is>
       </c>
-      <c r="C15" s="18" t="n">
+      <c r="C15" s="19" t="n">
         <v>15900</v>
       </c>
-      <c r="D15" s="18" t="n">
+      <c r="D15" s="19" t="n">
         <v>15400</v>
       </c>
-      <c r="E15" s="18" t="n">
+      <c r="E15" s="19" t="n">
         <v>13700</v>
       </c>
-      <c r="F15" s="18" t="n"/>
-      <c r="G15" s="18" t="n"/>
-      <c r="H15" s="18" t="n"/>
-      <c r="I15" s="18" t="n"/>
-      <c r="J15" s="18" t="n"/>
-      <c r="K15" s="18" t="n"/>
-      <c r="L15" s="18" t="n"/>
-      <c r="M15" s="18" t="n"/>
-      <c r="N15" s="18" t="n"/>
-      <c r="O15" s="19">
+      <c r="F15" s="19" t="n"/>
+      <c r="G15" s="19" t="n"/>
+      <c r="H15" s="19" t="n"/>
+      <c r="I15" s="19" t="n"/>
+      <c r="J15" s="19" t="n"/>
+      <c r="K15" s="19" t="n"/>
+      <c r="L15" s="19" t="n"/>
+      <c r="M15" s="19" t="n"/>
+      <c r="N15" s="19" t="n"/>
+      <c r="O15" s="20">
         <f>IF(COUNT(C15:N15)=0,"",AVERAGE(C15:N15))</f>
         <v/>
       </c>
-      <c r="P15" s="19">
+      <c r="P15" s="20">
         <f>IF(COUNT(C15:N15)=0,"",MAX(C15:N15))</f>
         <v/>
       </c>
-      <c r="Q15" s="19">
+      <c r="Q15" s="20">
         <f>IF(COUNT(C15:N15)=0,"",MIN(C15:N15))</f>
         <v/>
       </c>
@@ -1469,63 +1469,63 @@
           <t>% visitas → checkout</t>
         </is>
       </c>
-      <c r="C18" s="23">
+      <c r="C18" s="24">
         <f>IF(COUNT(C7:C15)&lt;9,"",IF(C8=0,0,C9/C8))</f>
         <v/>
       </c>
-      <c r="D18" s="23">
+      <c r="D18" s="24">
         <f>IF(COUNT(D7:D15)&lt;9,"",IF(D8=0,0,D9/D8))</f>
         <v/>
       </c>
-      <c r="E18" s="23">
+      <c r="E18" s="24">
         <f>IF(COUNT(E7:E15)&lt;9,"",IF(E8=0,0,E9/E8))</f>
         <v/>
       </c>
-      <c r="F18" s="23">
+      <c r="F18" s="24">
         <f>IF(COUNT(F7:F15)&lt;9,"",IF(F8=0,0,F9/F8))</f>
         <v/>
       </c>
-      <c r="G18" s="23">
+      <c r="G18" s="24">
         <f>IF(COUNT(G7:G15)&lt;9,"",IF(G8=0,0,G9/G8))</f>
         <v/>
       </c>
-      <c r="H18" s="23">
+      <c r="H18" s="24">
         <f>IF(COUNT(H7:H15)&lt;9,"",IF(H8=0,0,H9/H8))</f>
         <v/>
       </c>
-      <c r="I18" s="23">
+      <c r="I18" s="24">
         <f>IF(COUNT(I7:I15)&lt;9,"",IF(I8=0,0,I9/I8))</f>
         <v/>
       </c>
-      <c r="J18" s="23">
+      <c r="J18" s="24">
         <f>IF(COUNT(J7:J15)&lt;9,"",IF(J8=0,0,J9/J8))</f>
         <v/>
       </c>
-      <c r="K18" s="23">
+      <c r="K18" s="24">
         <f>IF(COUNT(K7:K15)&lt;9,"",IF(K8=0,0,K9/K8))</f>
         <v/>
       </c>
-      <c r="L18" s="23">
+      <c r="L18" s="24">
         <f>IF(COUNT(L7:L15)&lt;9,"",IF(L8=0,0,L9/L8))</f>
         <v/>
       </c>
-      <c r="M18" s="23">
+      <c r="M18" s="24">
         <f>IF(COUNT(M7:M15)&lt;9,"",IF(M8=0,0,M9/M8))</f>
         <v/>
       </c>
-      <c r="N18" s="23">
+      <c r="N18" s="24">
         <f>IF(COUNT(N7:N15)&lt;9,"",IF(N8=0,0,N9/N8))</f>
         <v/>
       </c>
-      <c r="O18" s="23">
+      <c r="O18" s="24">
         <f>IF(COUNT(C18:N18)=0,"",AVERAGE(C18:N18))</f>
         <v/>
       </c>
-      <c r="P18" s="23">
+      <c r="P18" s="24">
         <f>IF(COUNT(C18:N18)=0,"",MAX(C18:N18))</f>
         <v/>
       </c>
-      <c r="Q18" s="23">
+      <c r="Q18" s="24">
         <f>IF(COUNT(C18:N18)=0,"",MIN(C18:N18))</f>
         <v/>
       </c>
@@ -1536,63 +1536,63 @@
           <t>% checkout → compra</t>
         </is>
       </c>
-      <c r="C19" s="23">
+      <c r="C19" s="24">
         <f>IF(COUNT(C7:C15)&lt;9,"",IF(C9=0,0,C10/C9))</f>
         <v/>
       </c>
-      <c r="D19" s="23">
+      <c r="D19" s="24">
         <f>IF(COUNT(D7:D15)&lt;9,"",IF(D9=0,0,D10/D9))</f>
         <v/>
       </c>
-      <c r="E19" s="23">
+      <c r="E19" s="24">
         <f>IF(COUNT(E7:E15)&lt;9,"",IF(E9=0,0,E10/E9))</f>
         <v/>
       </c>
-      <c r="F19" s="23">
+      <c r="F19" s="24">
         <f>IF(COUNT(F7:F15)&lt;9,"",IF(F9=0,0,F10/F9))</f>
         <v/>
       </c>
-      <c r="G19" s="23">
+      <c r="G19" s="24">
         <f>IF(COUNT(G7:G15)&lt;9,"",IF(G9=0,0,G10/G9))</f>
         <v/>
       </c>
-      <c r="H19" s="23">
+      <c r="H19" s="24">
         <f>IF(COUNT(H7:H15)&lt;9,"",IF(H9=0,0,H10/H9))</f>
         <v/>
       </c>
-      <c r="I19" s="23">
+      <c r="I19" s="24">
         <f>IF(COUNT(I7:I15)&lt;9,"",IF(I9=0,0,I10/I9))</f>
         <v/>
       </c>
-      <c r="J19" s="23">
+      <c r="J19" s="24">
         <f>IF(COUNT(J7:J15)&lt;9,"",IF(J9=0,0,J10/J9))</f>
         <v/>
       </c>
-      <c r="K19" s="23">
+      <c r="K19" s="24">
         <f>IF(COUNT(K7:K15)&lt;9,"",IF(K9=0,0,K10/K9))</f>
         <v/>
       </c>
-      <c r="L19" s="23">
+      <c r="L19" s="24">
         <f>IF(COUNT(L7:L15)&lt;9,"",IF(L9=0,0,L10/L9))</f>
         <v/>
       </c>
-      <c r="M19" s="23">
+      <c r="M19" s="24">
         <f>IF(COUNT(M7:M15)&lt;9,"",IF(M9=0,0,M10/M9))</f>
         <v/>
       </c>
-      <c r="N19" s="23">
+      <c r="N19" s="24">
         <f>IF(COUNT(N7:N15)&lt;9,"",IF(N9=0,0,N10/N9))</f>
         <v/>
       </c>
-      <c r="O19" s="23">
+      <c r="O19" s="24">
         <f>IF(COUNT(C19:N19)=0,"",AVERAGE(C19:N19))</f>
         <v/>
       </c>
-      <c r="P19" s="23">
+      <c r="P19" s="24">
         <f>IF(COUNT(C19:N19)=0,"",MAX(C19:N19))</f>
         <v/>
       </c>
-      <c r="Q19" s="23">
+      <c r="Q19" s="24">
         <f>IF(COUNT(C19:N19)=0,"",MIN(C19:N19))</f>
         <v/>
       </c>
@@ -1852,15 +1852,15 @@
         <f>IF(COUNT(N7:N15)&lt;9,"",N14*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)-N8*'Supuestos'!$C$36-'Supuestos'!$C$37-N7)</f>
         <v/>
       </c>
-      <c r="O23" s="19">
+      <c r="O23" s="20">
         <f>IF(COUNT(C23:N23)=0,"",AVERAGE(C23:N23))</f>
         <v/>
       </c>
-      <c r="P23" s="19">
+      <c r="P23" s="20">
         <f>IF(COUNT(C23:N23)=0,"",MAX(C23:N23))</f>
         <v/>
       </c>
-      <c r="Q23" s="19">
+      <c r="Q23" s="20">
         <f>IF(COUNT(C23:N23)=0,"",MIN(C23:N23))</f>
         <v/>
       </c>
@@ -1871,63 +1871,63 @@
           <t>Ganancia de caja del período (con lo cobrado hasta ahora)</t>
         </is>
       </c>
-      <c r="C24" s="19">
+      <c r="C24" s="20">
         <f>IF(COUNT(C7:C15)&lt;9,"",C15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)-C8*'Supuestos'!$C$36-'Supuestos'!$C$37-C7)</f>
         <v/>
       </c>
-      <c r="D24" s="19">
+      <c r="D24" s="20">
         <f>IF(COUNT(D7:D15)&lt;9,"",D15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)-D8*'Supuestos'!$C$36-'Supuestos'!$C$37-D7)</f>
         <v/>
       </c>
-      <c r="E24" s="19">
+      <c r="E24" s="20">
         <f>IF(COUNT(E7:E15)&lt;9,"",E15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)-E8*'Supuestos'!$C$36-'Supuestos'!$C$37-E7)</f>
         <v/>
       </c>
-      <c r="F24" s="19">
+      <c r="F24" s="20">
         <f>IF(COUNT(F7:F15)&lt;9,"",F15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)-F8*'Supuestos'!$C$36-'Supuestos'!$C$37-F7)</f>
         <v/>
       </c>
-      <c r="G24" s="19">
+      <c r="G24" s="20">
         <f>IF(COUNT(G7:G15)&lt;9,"",G15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)-G8*'Supuestos'!$C$36-'Supuestos'!$C$37-G7)</f>
         <v/>
       </c>
-      <c r="H24" s="19">
+      <c r="H24" s="20">
         <f>IF(COUNT(H7:H15)&lt;9,"",H15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)-H8*'Supuestos'!$C$36-'Supuestos'!$C$37-H7)</f>
         <v/>
       </c>
-      <c r="I24" s="19">
+      <c r="I24" s="20">
         <f>IF(COUNT(I7:I15)&lt;9,"",I15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)-I8*'Supuestos'!$C$36-'Supuestos'!$C$37-I7)</f>
         <v/>
       </c>
-      <c r="J24" s="19">
+      <c r="J24" s="20">
         <f>IF(COUNT(J7:J15)&lt;9,"",J15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)-J8*'Supuestos'!$C$36-'Supuestos'!$C$37-J7)</f>
         <v/>
       </c>
-      <c r="K24" s="19">
+      <c r="K24" s="20">
         <f>IF(COUNT(K7:K15)&lt;9,"",K15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)-K8*'Supuestos'!$C$36-'Supuestos'!$C$37-K7)</f>
         <v/>
       </c>
-      <c r="L24" s="19">
+      <c r="L24" s="20">
         <f>IF(COUNT(L7:L15)&lt;9,"",L15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)-L8*'Supuestos'!$C$36-'Supuestos'!$C$37-L7)</f>
         <v/>
       </c>
-      <c r="M24" s="19">
+      <c r="M24" s="20">
         <f>IF(COUNT(M7:M15)&lt;9,"",M15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)-M8*'Supuestos'!$C$36-'Supuestos'!$C$37-M7)</f>
         <v/>
       </c>
-      <c r="N24" s="19">
+      <c r="N24" s="20">
         <f>IF(COUNT(N7:N15)&lt;9,"",N15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)-N8*'Supuestos'!$C$36-'Supuestos'!$C$37-N7)</f>
         <v/>
       </c>
-      <c r="O24" s="19">
+      <c r="O24" s="20">
         <f>IF(COUNT(C24:N24)=0,"",AVERAGE(C24:N24))</f>
         <v/>
       </c>
-      <c r="P24" s="19">
+      <c r="P24" s="20">
         <f>IF(COUNT(C24:N24)=0,"",MAX(C24:N24))</f>
         <v/>
       </c>
-      <c r="Q24" s="19">
+      <c r="Q24" s="20">
         <f>IF(COUNT(C24:N24)=0,"",MIN(C24:N24))</f>
         <v/>
       </c>
@@ -2053,15 +2053,15 @@
         <f>IF(COUNT(N7:N15)&lt;9,"",IF(N7=0,0,N14*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)/N7))</f>
         <v/>
       </c>
-      <c r="O26" s="26">
+      <c r="O26" s="27">
         <f>IF(COUNT(C26:N26)=0,"",AVERAGE(C26:N26))</f>
         <v/>
       </c>
-      <c r="P26" s="26">
+      <c r="P26" s="27">
         <f>IF(COUNT(C26:N26)=0,"",MAX(C26:N26))</f>
         <v/>
       </c>
-      <c r="Q26" s="26">
+      <c r="Q26" s="27">
         <f>IF(COUNT(C26:N26)=0,"",MIN(C26:N26))</f>
         <v/>
       </c>
@@ -2072,63 +2072,63 @@
           <t>ROAS de caja (cobrado hasta ahora)</t>
         </is>
       </c>
-      <c r="C27" s="26">
+      <c r="C27" s="27">
         <f>IF(COUNT(C7:C15)&lt;9,"",IF(C7=0,0,C15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)/C7))</f>
         <v/>
       </c>
-      <c r="D27" s="26">
+      <c r="D27" s="27">
         <f>IF(COUNT(D7:D15)&lt;9,"",IF(D7=0,0,D15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)/D7))</f>
         <v/>
       </c>
-      <c r="E27" s="26">
+      <c r="E27" s="27">
         <f>IF(COUNT(E7:E15)&lt;9,"",IF(E7=0,0,E15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)/E7))</f>
         <v/>
       </c>
-      <c r="F27" s="26">
+      <c r="F27" s="27">
         <f>IF(COUNT(F7:F15)&lt;9,"",IF(F7=0,0,F15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)/F7))</f>
         <v/>
       </c>
-      <c r="G27" s="26">
+      <c r="G27" s="27">
         <f>IF(COUNT(G7:G15)&lt;9,"",IF(G7=0,0,G15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)/G7))</f>
         <v/>
       </c>
-      <c r="H27" s="26">
+      <c r="H27" s="27">
         <f>IF(COUNT(H7:H15)&lt;9,"",IF(H7=0,0,H15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)/H7))</f>
         <v/>
       </c>
-      <c r="I27" s="26">
+      <c r="I27" s="27">
         <f>IF(COUNT(I7:I15)&lt;9,"",IF(I7=0,0,I15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)/I7))</f>
         <v/>
       </c>
-      <c r="J27" s="26">
+      <c r="J27" s="27">
         <f>IF(COUNT(J7:J15)&lt;9,"",IF(J7=0,0,J15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)/J7))</f>
         <v/>
       </c>
-      <c r="K27" s="26">
+      <c r="K27" s="27">
         <f>IF(COUNT(K7:K15)&lt;9,"",IF(K7=0,0,K15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)/K7))</f>
         <v/>
       </c>
-      <c r="L27" s="26">
+      <c r="L27" s="27">
         <f>IF(COUNT(L7:L15)&lt;9,"",IF(L7=0,0,L15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)/L7))</f>
         <v/>
       </c>
-      <c r="M27" s="26">
+      <c r="M27" s="27">
         <f>IF(COUNT(M7:M15)&lt;9,"",IF(M7=0,0,M15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)/M7))</f>
         <v/>
       </c>
-      <c r="N27" s="26">
+      <c r="N27" s="27">
         <f>IF(COUNT(N7:N15)&lt;9,"",IF(N7=0,0,N15*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35)/N7))</f>
         <v/>
       </c>
-      <c r="O27" s="26">
+      <c r="O27" s="27">
         <f>IF(COUNT(C27:N27)=0,"",AVERAGE(C27:N27))</f>
         <v/>
       </c>
-      <c r="P27" s="26">
+      <c r="P27" s="27">
         <f>IF(COUNT(C27:N27)=0,"",MAX(C27:N27))</f>
         <v/>
       </c>
-      <c r="Q27" s="26">
+      <c r="Q27" s="27">
         <f>IF(COUNT(C27:N27)=0,"",MIN(C27:N27))</f>
         <v/>
       </c>
@@ -2418,7 +2418,7 @@
           <t>&gt;5 %</t>
         </is>
       </c>
-      <c r="G7" s="23">
+      <c r="G7" s="24">
         <f>'Supuestos'!$C$12</f>
         <v/>
       </c>
@@ -2454,7 +2454,7 @@
           <t>&gt;30 %</t>
         </is>
       </c>
-      <c r="G8" s="23">
+      <c r="G8" s="24">
         <f>'Supuestos'!$C$13</f>
         <v/>
       </c>
@@ -2490,7 +2490,7 @@
           <t>&gt;1,5 %</t>
         </is>
       </c>
-      <c r="G9" s="25">
+      <c r="G9" s="26">
         <f>'Modelo'!$C$11</f>
         <v/>
       </c>
@@ -2526,7 +2526,7 @@
           <t>&gt;35 %</t>
         </is>
       </c>
-      <c r="G10" s="23">
+      <c r="G10" s="24">
         <f>'Supuestos'!$C$18</f>
         <v/>
       </c>
@@ -2562,7 +2562,7 @@
           <t>&gt;14 %</t>
         </is>
       </c>
-      <c r="G11" s="23">
+      <c r="G11" s="24">
         <f>'Supuestos'!$C$22</f>
         <v/>
       </c>
@@ -2598,7 +2598,7 @@
           <t>&gt;4 %</t>
         </is>
       </c>
-      <c r="G12" s="23">
+      <c r="G12" s="24">
         <f>'Supuestos'!$C$30</f>
         <v/>
       </c>
@@ -2634,7 +2634,7 @@
           <t>&gt;1,7</t>
         </is>
       </c>
-      <c r="G13" s="26">
+      <c r="G13" s="27">
         <f>'Modelo'!$C$31</f>
         <v/>
       </c>
@@ -2670,7 +2670,7 @@
           <t>&gt;2,5</t>
         </is>
       </c>
-      <c r="G14" s="26">
+      <c r="G14" s="27">
         <f>'Modelo'!$C$43</f>
         <v/>
       </c>
@@ -2706,7 +2706,7 @@
           <t>&lt;4 %</t>
         </is>
       </c>
-      <c r="G15" s="23">
+      <c r="G15" s="24">
         <f>'Supuestos'!$C$35</f>
         <v/>
       </c>
@@ -3413,7 +3413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -3466,7 +3466,7 @@
           <t>Ninguna celda con error en Modelo</t>
         </is>
       </c>
-      <c r="C6" s="36">
+      <c r="C6" s="18">
         <f>IF(ISERROR(SUM('Modelo'!C5:C160)),"REVISAR","OK")</f>
         <v/>
       </c>
@@ -3482,7 +3482,7 @@
           <t>Ninguna celda con error en Simulador</t>
         </is>
       </c>
-      <c r="C7" s="36">
+      <c r="C7" s="18">
         <f>IF(ISERROR(SUM('Simulador'!C5:G220)),"REVISAR","OK")</f>
         <v/>
       </c>
@@ -3498,7 +3498,7 @@
           <t>Ninguna celda con error en Embudo</t>
         </is>
       </c>
-      <c r="C8" s="36">
+      <c r="C8" s="18">
         <f>IF(ISERROR(SUM('Embudo'!C5:H60)),"REVISAR","OK")</f>
         <v/>
       </c>
@@ -3514,7 +3514,7 @@
           <t>Ninguna celda con error en Resumen</t>
         </is>
       </c>
-      <c r="C9" s="36">
+      <c r="C9" s="18">
         <f>IF(ISERROR(SUM('Resumen'!C5:C60)),"REVISAR","OK")</f>
         <v/>
       </c>
@@ -3530,7 +3530,7 @@
           <t>Ninguna celda con error en Proyección 12 meses</t>
         </is>
       </c>
-      <c r="C10" s="36">
+      <c r="C10" s="18">
         <f>IF(ISERROR(SUM('Proyección 12 meses'!C5:O40)),"REVISAR","OK")</f>
         <v/>
       </c>
@@ -3546,7 +3546,7 @@
           <t>Ninguna celda con error en Escenarios</t>
         </is>
       </c>
-      <c r="C11" s="36">
+      <c r="C11" s="18">
         <f>IF(ISERROR(SUM('Escenarios'!C5:L120)),"REVISAR","OK")</f>
         <v/>
       </c>
@@ -3562,7 +3562,7 @@
           <t>Ninguna celda con error en Seguimiento</t>
         </is>
       </c>
-      <c r="C12" s="36">
+      <c r="C12" s="18">
         <f>IF(ISERROR(SUM('Seguimiento'!C5:Q80)),"REVISAR","OK")</f>
         <v/>
       </c>
@@ -3578,7 +3578,7 @@
           <t>Los supuestos de tráfico son mayores a cero</t>
         </is>
       </c>
-      <c r="C13" s="36">
+      <c r="C13" s="18">
         <f>IF(AND('Supuestos'!$C$9&gt;0,'Supuestos'!$C$12&gt;0,'Supuestos'!$C$13&gt;0),"OK","REVISAR")</f>
         <v/>
       </c>
@@ -3594,7 +3594,7 @@
           <t>La curva de cobranza suma 100 %</t>
         </is>
       </c>
-      <c r="C14" s="36">
+      <c r="C14" s="18">
         <f>IF(ABS('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42-1)&lt;0.001,"OK","REVISAR")</f>
         <v/>
       </c>
@@ -3610,7 +3610,7 @@
           <t>Comisiones + reembolsos menores al 60 %</t>
         </is>
       </c>
-      <c r="C15" s="36">
+      <c r="C15" s="18">
         <f>IF(('Supuestos'!$C$33+'Supuestos'!$C$34+'Supuestos'!$C$35)&lt;0.6,"OK","REVISAR")</f>
         <v/>
       </c>
@@ -3626,7 +3626,7 @@
           <t>El escenario en uso es 1, 2 o 3</t>
         </is>
       </c>
-      <c r="C16" s="36">
+      <c r="C16" s="18">
         <f>IF(OR('Supuestos'!$C$6=1,'Supuestos'!$C$6=2,'Supuestos'!$C$6=3),"OK","REVISAR")</f>
         <v/>
       </c>
@@ -3642,7 +3642,7 @@
           <t>La inversión es mayor a cero</t>
         </is>
       </c>
-      <c r="C17" s="36">
+      <c r="C17" s="18">
         <f>IF('Supuestos'!$C$8&gt;0,"OK","REVISAR")</f>
         <v/>
       </c>
@@ -3654,7 +3654,7 @@
           <t>La meta de ventas es alcanzable (hay conversión a venta)</t>
         </is>
       </c>
-      <c r="C18" s="36">
+      <c r="C18" s="18">
         <f>IF('Modelo'!$C$11&gt;0,"OK","REVISAR")</f>
         <v/>
       </c>
@@ -3670,7 +3670,7 @@
           <t>Las conversiones están entre 0 y 100 %</t>
         </is>
       </c>
-      <c r="C19" s="36">
+      <c r="C19" s="18">
         <f>IF(AND('Supuestos'!$C$12&gt;=0,'Supuestos'!$C$12&lt;=1,'Supuestos'!$C$13&gt;=0,'Supuestos'!$C$13&lt;=1,'Supuestos'!$C$18&gt;=0,'Supuestos'!$C$18&lt;=1,'Supuestos'!$C$20&gt;=0,'Supuestos'!$C$20&lt;=1,'Supuestos'!$C$22&gt;=0,'Supuestos'!$C$22&lt;=1,'Supuestos'!$C$24&gt;=0,'Supuestos'!$C$24&lt;=1,'Supuestos'!$C$26&gt;=0,'Supuestos'!$C$26&lt;=1,'Supuestos'!$C$28&gt;=0,'Supuestos'!$C$28&lt;=1,'Supuestos'!$C$30&gt;=0,'Supuestos'!$C$30&lt;=1),"OK","REVISAR")</f>
         <v/>
       </c>
@@ -3686,7 +3686,7 @@
           <t>El margen de seguridad está entre 0 y 100 %</t>
         </is>
       </c>
-      <c r="C20" s="36">
+      <c r="C20" s="18">
         <f>IF(AND('Supuestos'!$C$46&gt;=0,'Supuestos'!$C$46&lt;=1),"OK","REVISAR")</f>
         <v/>
       </c>
@@ -3698,7 +3698,7 @@
           <t>El crecimiento mensual está entre −50 % y 100 %</t>
         </is>
       </c>
-      <c r="C21" s="36">
+      <c r="C21" s="18">
         <f>IF(AND('Supuestos'!$C$48&gt;=-0.5,'Supuestos'!$C$48&lt;=1),"OK","REVISAR")</f>
         <v/>
       </c>
@@ -3714,7 +3714,7 @@
           <t>La cadena es decreciente (cada etapa tiene menos gente que la anterior)</t>
         </is>
       </c>
-      <c r="C22" s="36">
+      <c r="C22" s="18">
         <f>IF(AND('Modelo'!$C$9&lt;='Modelo'!$C$8,'Modelo'!$C$10&lt;='Modelo'!$C$9),"OK","REVISAR")</f>
         <v/>
       </c>
@@ -3724,19 +3724,196 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Simulador: lo que escribiste en las celdas amarillas</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="8" t="n"/>
+    </row>
     <row r="24">
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Ningún supuesto del Simulador fuera de rango (porcentajes entre 0 y 1, números no negativos)</t>
+        </is>
+      </c>
+      <c r="C24" s="18">
+        <f>IF(COUNTIF('Simulador'!$I$6:$I$93,"REVISAR")=0,"OK","REVISAR")</f>
+        <v/>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>La columna Rango del Simulador marca la fila con el problema.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Simulador: Los supuestos de tráfico son mayores a cero</t>
+        </is>
+      </c>
+      <c r="C25" s="18">
+        <f>IF(AND('Simulador'!$C$7&gt;0,'Simulador'!$C$11&gt;0,'Simulador'!$C$13&gt;0),"OK","REVISAR")</f>
+        <v/>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Con un 0 en el tráfico o en la conversión de la página no hay unidades y el modelo no dice nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Simulador: La curva de cobranza suma 100 %</t>
+        </is>
+      </c>
+      <c r="C26" s="18">
+        <f>IF(ABS('Simulador'!$C$54+'Simulador'!$C$55+'Simulador'!$C$56-1)&lt;0.001,"OK","REVISAR")</f>
+        <v/>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Supuestos → cobranza mes 1 + mes 2 + mes 3 = 100 %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Simulador: Comisiones + reembolsos menores al 60 %</t>
+        </is>
+      </c>
+      <c r="C27" s="18">
+        <f>IF(('Simulador'!$C$59+'Simulador'!$C$60+'Simulador'!$C$62)&lt;0.6,"OK","REVISAR")</f>
+        <v/>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Si suman más, revisá los porcentajes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Simulador: El escenario en uso es 1, 2 o 3</t>
+        </is>
+      </c>
+      <c r="C28" s="18">
+        <f>IF(OR('Supuestos'!$C$6=1,'Supuestos'!$C$6=2,'Supuestos'!$C$6=3),"OK","REVISAR")</f>
+        <v/>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Supuestos → celda 'Escenario en uso'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Simulador: La inversión es mayor a cero</t>
+        </is>
+      </c>
+      <c r="C29" s="18">
+        <f>IF('Simulador'!$C$9&gt;0,"OK","REVISAR")</f>
+        <v/>
+      </c>
+      <c r="D29" s="5" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Simulador: La meta de ventas es alcanzable (hay conversión a venta)</t>
+        </is>
+      </c>
+      <c r="C30" s="18">
+        <f>IF('Simulador'!$E$15&gt;0,"OK","REVISAR")</f>
+        <v/>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Con conversión a venta en 0, la inversión para la meta dice 'inalcanzable con estos supuestos'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Simulador: Las conversiones están entre 0 y 100 %</t>
+        </is>
+      </c>
+      <c r="C31" s="18">
+        <f>IF(AND('Simulador'!$C$11&gt;=0,'Simulador'!$C$11&lt;=1,'Simulador'!$C$13&gt;=0,'Simulador'!$C$13&lt;=1,'Simulador'!$C$20&gt;=0,'Simulador'!$C$20&lt;=1,'Simulador'!$C$24&gt;=0,'Simulador'!$C$24&lt;=1,'Simulador'!$C$28&gt;=0,'Simulador'!$C$28&lt;=1,'Simulador'!$C$32&gt;=0,'Simulador'!$C$32&lt;=1,'Simulador'!$C$36&gt;=0,'Simulador'!$C$36&lt;=1,'Simulador'!$C$40&gt;=0,'Simulador'!$C$40&lt;=1,'Simulador'!$C$44&gt;=0,'Simulador'!$C$44&lt;=1),"OK","REVISAR")</f>
+        <v/>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Un 25 % se escribe 25 % (o 0,25), no 25.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Simulador: El margen de seguridad está entre 0 y 100 %</t>
+        </is>
+      </c>
+      <c r="C32" s="18">
+        <f>IF(AND('Simulador'!$C$77&gt;=0,'Simulador'!$C$77&lt;=1),"OK","REVISAR")</f>
+        <v/>
+      </c>
+      <c r="D32" s="5" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Simulador: El crecimiento mensual está entre −50 % y 100 %</t>
+        </is>
+      </c>
+      <c r="C33" s="18">
+        <f>IF(AND('Supuestos'!$C$48&gt;=-0.5,'Supuestos'!$C$48&lt;=1),"OK","REVISAR")</f>
+        <v/>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Más de 100 % por mes no es realista para una proyección.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Simulador: La cadena es decreciente (cada etapa tiene menos gente que la anterior)</t>
+        </is>
+      </c>
+      <c r="C34" s="18">
+        <f>IF(AND('Simulador'!$E$12&lt;='Simulador'!$E$10,'Simulador'!$E$14&lt;='Simulador'!$E$12),"OK","REVISAR")</f>
+        <v/>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Si falla, alguna conversión está por encima de 100 %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>Estado general del modelo</t>
         </is>
       </c>
-      <c r="C24" s="37">
-        <f>IF(COUNTIF(C6:C22,"REVISAR")=0,"OK","REVISAR")</f>
+      <c r="C36" s="37">
+        <f>IF(COUNTIF(C6:C34,"REVISAR")=0,"OK","REVISAR")</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C6:C24">
+  <conditionalFormatting sqref="C6:C36">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"OK"</formula>
     </cfRule>
@@ -4332,7 +4509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H97"/>
+  <dimension ref="A1:I98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -4343,6 +4520,7 @@
     <col width="19" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="62" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4400,6 +4578,11 @@
       <c r="H5" s="6" t="inlineStr">
         <is>
           <t>Cómo se calcula</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>Rango</t>
         </is>
       </c>
     </row>
@@ -4439,6 +4622,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I7" s="18">
+        <f>IF(AND(ISNUMBER(C7),C7&gt;=0),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="B8" t="inlineStr">
@@ -4470,11 +4657,11 @@
           <t>Inversión en publicidad por mes</t>
         </is>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="19">
         <f>'Supuestos'!$C$8</f>
         <v/>
       </c>
-      <c r="D9" s="19">
+      <c r="D9" s="20">
         <f>'Supuestos'!$C$8</f>
         <v/>
       </c>
@@ -4487,6 +4674,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I9" s="18">
+        <f>IF(AND(ISNUMBER(C9),C9&gt;=0),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="4" t="inlineStr">
@@ -4494,15 +4685,15 @@
           <t>Visitas a la página de ventas</t>
         </is>
       </c>
-      <c r="E10" s="20">
+      <c r="E10" s="21">
         <f>IF($E$8=0,0,$C$9/$E$8)</f>
         <v/>
       </c>
-      <c r="F10" s="21">
+      <c r="F10" s="22">
         <f>'Modelo'!$C$8</f>
         <v/>
       </c>
-      <c r="G10" s="21">
+      <c r="G10" s="22">
         <f>IF(AND(ISNUMBER(E10),ISNUMBER(F10)),E10-F10,"")</f>
         <v/>
       </c>
@@ -4518,11 +4709,11 @@
           <t>% de visitas que llegan al checkout</t>
         </is>
       </c>
-      <c r="C11" s="22">
+      <c r="C11" s="23">
         <f>'Supuestos'!$C$12</f>
         <v/>
       </c>
-      <c r="D11" s="23">
+      <c r="D11" s="24">
         <f>'Supuestos'!$C$12</f>
         <v/>
       </c>
@@ -4535,6 +4726,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I11" s="18">
+        <f>IF(AND(ISNUMBER(C11),C11&gt;=0,C11&lt;=1),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="B12" t="inlineStr">
@@ -4542,15 +4737,15 @@
           <t>Checkouts iniciados</t>
         </is>
       </c>
-      <c r="E12" s="21">
+      <c r="E12" s="22">
         <f>$E$10*$C$11</f>
         <v/>
       </c>
-      <c r="F12" s="21">
+      <c r="F12" s="22">
         <f>'Modelo'!$C$9</f>
         <v/>
       </c>
-      <c r="G12" s="21">
+      <c r="G12" s="22">
         <f>IF(AND(ISNUMBER(E12),ISNUMBER(F12)),E12-F12,"")</f>
         <v/>
       </c>
@@ -4566,11 +4761,11 @@
           <t>% de checkouts que terminan en compra</t>
         </is>
       </c>
-      <c r="C13" s="22">
+      <c r="C13" s="23">
         <f>'Supuestos'!$C$13</f>
         <v/>
       </c>
-      <c r="D13" s="23">
+      <c r="D13" s="24">
         <f>'Supuestos'!$C$13</f>
         <v/>
       </c>
@@ -4583,6 +4778,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I13" s="18">
+        <f>IF(AND(ISNUMBER(C13),C13&gt;=0,C13&lt;=1),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="4" t="inlineStr">
@@ -4594,11 +4793,11 @@
         <f>$E$12*$C$13</f>
         <v/>
       </c>
-      <c r="F14" s="24">
+      <c r="F14" s="25">
         <f>'Modelo'!$C$10</f>
         <v/>
       </c>
-      <c r="G14" s="24">
+      <c r="G14" s="25">
         <f>IF(AND(ISNUMBER(E14),ISNUMBER(F14)),E14-F14,"")</f>
         <v/>
       </c>
@@ -4614,15 +4813,15 @@
           <t>% de visitas que compran</t>
         </is>
       </c>
-      <c r="E15" s="25">
+      <c r="E15" s="26">
         <f>IF($E$10=0,0,$E$14/$E$10)</f>
         <v/>
       </c>
-      <c r="F15" s="25">
+      <c r="F15" s="26">
         <f>'Modelo'!$C$11</f>
         <v/>
       </c>
-      <c r="G15" s="25">
+      <c r="G15" s="26">
         <f>IF(AND(ISNUMBER(E15),ISNUMBER(F15)),E15-F15,"")</f>
         <v/>
       </c>
@@ -4692,6 +4891,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I18" s="18">
+        <f>IF(AND(ISNUMBER(C18),C18&gt;=0),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="B19" t="inlineStr">
@@ -4699,15 +4902,15 @@
           <t>Facturado: producto principal</t>
         </is>
       </c>
-      <c r="E19" s="19">
+      <c r="E19" s="20">
         <f>$E$14*$C$18</f>
         <v/>
       </c>
-      <c r="F19" s="19">
+      <c r="F19" s="20">
         <f>'Modelo'!$C$14</f>
         <v/>
       </c>
-      <c r="G19" s="19">
+      <c r="G19" s="20">
         <f>IF(AND(ISNUMBER(E19),ISNUMBER(F19)),E19-F19,"")</f>
         <v/>
       </c>
@@ -4723,11 +4926,11 @@
           <t>Bump 1: % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C20" s="22">
+      <c r="C20" s="23">
         <f>'Supuestos'!$C$18</f>
         <v/>
       </c>
-      <c r="D20" s="23">
+      <c r="D20" s="24">
         <f>'Supuestos'!$C$18</f>
         <v/>
       </c>
@@ -4740,6 +4943,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I20" s="18">
+        <f>IF(AND(ISNUMBER(C20),C20&gt;=0,C20&lt;=1),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="B21" t="inlineStr">
@@ -4747,15 +4954,15 @@
           <t>Ventas: Bump 1</t>
         </is>
       </c>
-      <c r="E21" s="24">
+      <c r="E21" s="25">
         <f>$E$14*$C$20</f>
         <v/>
       </c>
-      <c r="F21" s="24">
+      <c r="F21" s="25">
         <f>'Modelo'!$C$15</f>
         <v/>
       </c>
-      <c r="G21" s="24">
+      <c r="G21" s="25">
         <f>IF(AND(ISNUMBER(E21),ISNUMBER(F21)),E21-F21,"")</f>
         <v/>
       </c>
@@ -4788,6 +4995,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I22" s="18">
+        <f>IF(AND(ISNUMBER(C22),C22&gt;=0),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="B23" t="inlineStr">
@@ -4795,15 +5006,15 @@
           <t>Facturado: Bump 1</t>
         </is>
       </c>
-      <c r="E23" s="19">
+      <c r="E23" s="20">
         <f>$E$21*$C$22</f>
         <v/>
       </c>
-      <c r="F23" s="19">
+      <c r="F23" s="20">
         <f>'Modelo'!$C$16</f>
         <v/>
       </c>
-      <c r="G23" s="19">
+      <c r="G23" s="20">
         <f>IF(AND(ISNUMBER(E23),ISNUMBER(F23)),E23-F23,"")</f>
         <v/>
       </c>
@@ -4819,11 +5030,11 @@
           <t>Bump 2: % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C24" s="22">
+      <c r="C24" s="23">
         <f>'Supuestos'!$C$20</f>
         <v/>
       </c>
-      <c r="D24" s="23">
+      <c r="D24" s="24">
         <f>'Supuestos'!$C$20</f>
         <v/>
       </c>
@@ -4836,6 +5047,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I24" s="18">
+        <f>IF(AND(ISNUMBER(C24),C24&gt;=0,C24&lt;=1),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="B25" t="inlineStr">
@@ -4843,15 +5058,15 @@
           <t>Ventas: Bump 2</t>
         </is>
       </c>
-      <c r="E25" s="24">
+      <c r="E25" s="25">
         <f>$E$14*$C$24</f>
         <v/>
       </c>
-      <c r="F25" s="24">
+      <c r="F25" s="25">
         <f>'Modelo'!$C$17</f>
         <v/>
       </c>
-      <c r="G25" s="24">
+      <c r="G25" s="25">
         <f>IF(AND(ISNUMBER(E25),ISNUMBER(F25)),E25-F25,"")</f>
         <v/>
       </c>
@@ -4884,6 +5099,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I26" s="18">
+        <f>IF(AND(ISNUMBER(C26),C26&gt;=0),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="B27" t="inlineStr">
@@ -4891,15 +5110,15 @@
           <t>Facturado: Bump 2</t>
         </is>
       </c>
-      <c r="E27" s="19">
+      <c r="E27" s="20">
         <f>$E$25*$C$26</f>
         <v/>
       </c>
-      <c r="F27" s="19">
+      <c r="F27" s="20">
         <f>'Modelo'!$C$18</f>
         <v/>
       </c>
-      <c r="G27" s="19">
+      <c r="G27" s="20">
         <f>IF(AND(ISNUMBER(E27),ISNUMBER(F27)),E27-F27,"")</f>
         <v/>
       </c>
@@ -4915,11 +5134,11 @@
           <t>OTO 1: % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C28" s="22">
+      <c r="C28" s="23">
         <f>'Supuestos'!$C$22</f>
         <v/>
       </c>
-      <c r="D28" s="23">
+      <c r="D28" s="24">
         <f>'Supuestos'!$C$22</f>
         <v/>
       </c>
@@ -4932,6 +5151,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I28" s="18">
+        <f>IF(AND(ISNUMBER(C28),C28&gt;=0,C28&lt;=1),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="B29" t="inlineStr">
@@ -4939,15 +5162,15 @@
           <t>Ventas: OTO 1</t>
         </is>
       </c>
-      <c r="E29" s="24">
+      <c r="E29" s="25">
         <f>$E$14*$C$28</f>
         <v/>
       </c>
-      <c r="F29" s="24">
+      <c r="F29" s="25">
         <f>'Modelo'!$C$19</f>
         <v/>
       </c>
-      <c r="G29" s="24">
+      <c r="G29" s="25">
         <f>IF(AND(ISNUMBER(E29),ISNUMBER(F29)),E29-F29,"")</f>
         <v/>
       </c>
@@ -4980,6 +5203,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I30" s="18">
+        <f>IF(AND(ISNUMBER(C30),C30&gt;=0),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="B31" t="inlineStr">
@@ -4987,15 +5214,15 @@
           <t>Facturado: OTO 1</t>
         </is>
       </c>
-      <c r="E31" s="19">
+      <c r="E31" s="20">
         <f>$E$29*$C$30</f>
         <v/>
       </c>
-      <c r="F31" s="19">
+      <c r="F31" s="20">
         <f>'Modelo'!$C$20</f>
         <v/>
       </c>
-      <c r="G31" s="19">
+      <c r="G31" s="20">
         <f>IF(AND(ISNUMBER(E31),ISNUMBER(F31)),E31-F31,"")</f>
         <v/>
       </c>
@@ -5011,11 +5238,11 @@
           <t>OTO 2: % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C32" s="22">
+      <c r="C32" s="23">
         <f>'Supuestos'!$C$24</f>
         <v/>
       </c>
-      <c r="D32" s="23">
+      <c r="D32" s="24">
         <f>'Supuestos'!$C$24</f>
         <v/>
       </c>
@@ -5028,6 +5255,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I32" s="18">
+        <f>IF(AND(ISNUMBER(C32),C32&gt;=0,C32&lt;=1),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="B33" t="inlineStr">
@@ -5035,15 +5266,15 @@
           <t>Ventas: OTO 2</t>
         </is>
       </c>
-      <c r="E33" s="24">
+      <c r="E33" s="25">
         <f>$E$14*$C$32</f>
         <v/>
       </c>
-      <c r="F33" s="24">
+      <c r="F33" s="25">
         <f>'Modelo'!$C$21</f>
         <v/>
       </c>
-      <c r="G33" s="24">
+      <c r="G33" s="25">
         <f>IF(AND(ISNUMBER(E33),ISNUMBER(F33)),E33-F33,"")</f>
         <v/>
       </c>
@@ -5076,6 +5307,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I34" s="18">
+        <f>IF(AND(ISNUMBER(C34),C34&gt;=0),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="B35" t="inlineStr">
@@ -5083,15 +5318,15 @@
           <t>Facturado: OTO 2</t>
         </is>
       </c>
-      <c r="E35" s="19">
+      <c r="E35" s="20">
         <f>$E$33*$C$34</f>
         <v/>
       </c>
-      <c r="F35" s="19">
+      <c r="F35" s="20">
         <f>'Modelo'!$C$22</f>
         <v/>
       </c>
-      <c r="G35" s="19">
+      <c r="G35" s="20">
         <f>IF(AND(ISNUMBER(E35),ISNUMBER(F35)),E35-F35,"")</f>
         <v/>
       </c>
@@ -5107,11 +5342,11 @@
           <t>OTO 3: % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C36" s="22">
+      <c r="C36" s="23">
         <f>'Supuestos'!$C$26</f>
         <v/>
       </c>
-      <c r="D36" s="23">
+      <c r="D36" s="24">
         <f>'Supuestos'!$C$26</f>
         <v/>
       </c>
@@ -5124,6 +5359,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I36" s="18">
+        <f>IF(AND(ISNUMBER(C36),C36&gt;=0,C36&lt;=1),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="B37" t="inlineStr">
@@ -5131,15 +5370,15 @@
           <t>Ventas: OTO 3</t>
         </is>
       </c>
-      <c r="E37" s="24">
+      <c r="E37" s="25">
         <f>$E$14*$C$36</f>
         <v/>
       </c>
-      <c r="F37" s="24">
+      <c r="F37" s="25">
         <f>'Modelo'!$C$23</f>
         <v/>
       </c>
-      <c r="G37" s="24">
+      <c r="G37" s="25">
         <f>IF(AND(ISNUMBER(E37),ISNUMBER(F37)),E37-F37,"")</f>
         <v/>
       </c>
@@ -5172,6 +5411,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I38" s="18">
+        <f>IF(AND(ISNUMBER(C38),C38&gt;=0),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="B39" t="inlineStr">
@@ -5179,15 +5422,15 @@
           <t>Facturado: OTO 3</t>
         </is>
       </c>
-      <c r="E39" s="19">
+      <c r="E39" s="20">
         <f>$E$37*$C$38</f>
         <v/>
       </c>
-      <c r="F39" s="19">
+      <c r="F39" s="20">
         <f>'Modelo'!$C$24</f>
         <v/>
       </c>
-      <c r="G39" s="19">
+      <c r="G39" s="20">
         <f>IF(AND(ISNUMBER(E39),ISNUMBER(F39)),E39-F39,"")</f>
         <v/>
       </c>
@@ -5203,11 +5446,11 @@
           <t>OTO 4: % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C40" s="22">
+      <c r="C40" s="23">
         <f>'Supuestos'!$C$28</f>
         <v/>
       </c>
-      <c r="D40" s="23">
+      <c r="D40" s="24">
         <f>'Supuestos'!$C$28</f>
         <v/>
       </c>
@@ -5220,6 +5463,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I40" s="18">
+        <f>IF(AND(ISNUMBER(C40),C40&gt;=0,C40&lt;=1),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="B41" t="inlineStr">
@@ -5227,15 +5474,15 @@
           <t>Ventas: OTO 4</t>
         </is>
       </c>
-      <c r="E41" s="24">
+      <c r="E41" s="25">
         <f>$E$14*$C$40</f>
         <v/>
       </c>
-      <c r="F41" s="24">
+      <c r="F41" s="25">
         <f>'Modelo'!$C$25</f>
         <v/>
       </c>
-      <c r="G41" s="24">
+      <c r="G41" s="25">
         <f>IF(AND(ISNUMBER(E41),ISNUMBER(F41)),E41-F41,"")</f>
         <v/>
       </c>
@@ -5268,6 +5515,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I42" s="18">
+        <f>IF(AND(ISNUMBER(C42),C42&gt;=0),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="B43" t="inlineStr">
@@ -5275,15 +5526,15 @@
           <t>Facturado: OTO 4</t>
         </is>
       </c>
-      <c r="E43" s="19">
+      <c r="E43" s="20">
         <f>$E$41*$C$42</f>
         <v/>
       </c>
-      <c r="F43" s="19">
+      <c r="F43" s="20">
         <f>'Modelo'!$C$26</f>
         <v/>
       </c>
-      <c r="G43" s="19">
+      <c r="G43" s="20">
         <f>IF(AND(ISNUMBER(E43),ISNUMBER(F43)),E43-F43,"")</f>
         <v/>
       </c>
@@ -5299,11 +5550,11 @@
           <t>Ascensión (programa de mayor valor): % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C44" s="22">
+      <c r="C44" s="23">
         <f>'Supuestos'!$C$30</f>
         <v/>
       </c>
-      <c r="D44" s="23">
+      <c r="D44" s="24">
         <f>'Supuestos'!$C$30</f>
         <v/>
       </c>
@@ -5316,6 +5567,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I44" s="18">
+        <f>IF(AND(ISNUMBER(C44),C44&gt;=0,C44&lt;=1),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="B45" t="inlineStr">
@@ -5323,15 +5578,15 @@
           <t>Ventas: Ascensión (programa de mayor valor)</t>
         </is>
       </c>
-      <c r="E45" s="24">
+      <c r="E45" s="25">
         <f>$E$14*$C$44</f>
         <v/>
       </c>
-      <c r="F45" s="24">
+      <c r="F45" s="25">
         <f>'Modelo'!$C$27</f>
         <v/>
       </c>
-      <c r="G45" s="24">
+      <c r="G45" s="25">
         <f>IF(AND(ISNUMBER(E45),ISNUMBER(F45)),E45-F45,"")</f>
         <v/>
       </c>
@@ -5364,6 +5619,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I46" s="18">
+        <f>IF(AND(ISNUMBER(C46),C46&gt;=0),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="B47" t="inlineStr">
@@ -5371,15 +5630,15 @@
           <t>Facturado: Ascensión (programa de mayor valor)</t>
         </is>
       </c>
-      <c r="E47" s="19">
+      <c r="E47" s="20">
         <f>$E$45*$C$46</f>
         <v/>
       </c>
-      <c r="F47" s="19">
+      <c r="F47" s="20">
         <f>'Modelo'!$C$28</f>
         <v/>
       </c>
-      <c r="G47" s="19">
+      <c r="G47" s="20">
         <f>IF(AND(ISNUMBER(E47),ISNUMBER(F47)),E47-F47,"")</f>
         <v/>
       </c>
@@ -5399,11 +5658,11 @@
         <f>$E$19+$E$23+$E$27+$E$31+$E$35+$E$39+$E$43+$E$47</f>
         <v/>
       </c>
-      <c r="F48" s="19">
+      <c r="F48" s="20">
         <f>'Modelo'!$C$29</f>
         <v/>
       </c>
-      <c r="G48" s="19">
+      <c r="G48" s="20">
         <f>IF(AND(ISNUMBER(E48),ISNUMBER(F48)),E48-F48,"")</f>
         <v/>
       </c>
@@ -5443,15 +5702,15 @@
           <t>AOV ÷ precio del principal</t>
         </is>
       </c>
-      <c r="E50" s="26">
+      <c r="E50" s="27">
         <f>IF($C$18=0,0,$E$49/$C$18)</f>
         <v/>
       </c>
-      <c r="F50" s="26">
+      <c r="F50" s="27">
         <f>'Modelo'!$C$31</f>
         <v/>
       </c>
-      <c r="G50" s="26">
+      <c r="G50" s="27">
         <f>IF(AND(ISNUMBER(E50),ISNUMBER(F50)),E50-F50,"")</f>
         <v/>
       </c>
@@ -5467,15 +5726,15 @@
           <t>Ventas del principal por visita (para la proyección)</t>
         </is>
       </c>
-      <c r="E51" s="25">
+      <c r="E51" s="26">
         <f>IF($E$10=0,0,$E$14/$E$10)</f>
         <v/>
       </c>
-      <c r="F51" s="25">
+      <c r="F51" s="26">
         <f>'Modelo'!$C$32</f>
         <v/>
       </c>
-      <c r="G51" s="25">
+      <c r="G51" s="26">
         <f>IF(AND(ISNUMBER(E51),ISNUMBER(F51)),E51-F51,"")</f>
         <v/>
       </c>
@@ -5528,11 +5787,11 @@
           <t>% del facturado que entra en el mes 1</t>
         </is>
       </c>
-      <c r="C54" s="22">
+      <c r="C54" s="23">
         <f>'Supuestos'!$C$40</f>
         <v/>
       </c>
-      <c r="D54" s="23">
+      <c r="D54" s="24">
         <f>'Supuestos'!$C$40</f>
         <v/>
       </c>
@@ -5545,6 +5804,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I54" s="18">
+        <f>IF(AND(ISNUMBER(C54),C54&gt;=0,C54&lt;=1),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="B55" t="inlineStr">
@@ -5552,11 +5815,11 @@
           <t>% que entra en el mes 2</t>
         </is>
       </c>
-      <c r="C55" s="22">
+      <c r="C55" s="23">
         <f>'Supuestos'!$C$41</f>
         <v/>
       </c>
-      <c r="D55" s="23">
+      <c r="D55" s="24">
         <f>'Supuestos'!$C$41</f>
         <v/>
       </c>
@@ -5569,6 +5832,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I55" s="18">
+        <f>IF(AND(ISNUMBER(C55),C55&gt;=0,C55&lt;=1),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="B56" t="inlineStr">
@@ -5576,11 +5843,11 @@
           <t>% que entra en el mes 3</t>
         </is>
       </c>
-      <c r="C56" s="22">
+      <c r="C56" s="23">
         <f>'Supuestos'!$C$42</f>
         <v/>
       </c>
-      <c r="D56" s="23">
+      <c r="D56" s="24">
         <f>'Supuestos'!$C$42</f>
         <v/>
       </c>
@@ -5593,6 +5860,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I56" s="18">
+        <f>IF(AND(ISNUMBER(C56),C56&gt;=0,C56&lt;=1),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="B57" t="inlineStr">
@@ -5600,15 +5871,15 @@
           <t>Cash a cobrar (facturado × cobranza completa)</t>
         </is>
       </c>
-      <c r="E57" s="19">
+      <c r="E57" s="20">
         <f>$E$48*($C$54+$C$55+$C$56)</f>
         <v/>
       </c>
-      <c r="F57" s="19">
+      <c r="F57" s="20">
         <f>'Modelo'!$C$35</f>
         <v/>
       </c>
-      <c r="G57" s="19">
+      <c r="G57" s="20">
         <f>IF(AND(ISNUMBER(E57),ISNUMBER(F57)),E57-F57,"")</f>
         <v/>
       </c>
@@ -5624,15 +5895,15 @@
           <t>Cash que entra en el primer mes</t>
         </is>
       </c>
-      <c r="E58" s="19">
+      <c r="E58" s="20">
         <f>$E$48*$C$54</f>
         <v/>
       </c>
-      <c r="F58" s="19">
+      <c r="F58" s="20">
         <f>'Modelo'!$C$36</f>
         <v/>
       </c>
-      <c r="G58" s="19">
+      <c r="G58" s="20">
         <f>IF(AND(ISNUMBER(E58),ISNUMBER(F58)),E58-F58,"")</f>
         <v/>
       </c>
@@ -5648,11 +5919,11 @@
           <t>Comisión de la pasarela o plataforma de pago</t>
         </is>
       </c>
-      <c r="C59" s="22">
+      <c r="C59" s="23">
         <f>'Supuestos'!$C$33</f>
         <v/>
       </c>
-      <c r="D59" s="23">
+      <c r="D59" s="24">
         <f>'Supuestos'!$C$33</f>
         <v/>
       </c>
@@ -5665,6 +5936,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I59" s="18">
+        <f>IF(AND(ISNUMBER(C59),C59&gt;=0,C59&lt;=1),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="B60" t="inlineStr">
@@ -5672,11 +5947,11 @@
           <t>Comisión del equipo de ventas</t>
         </is>
       </c>
-      <c r="C60" s="22">
+      <c r="C60" s="23">
         <f>'Supuestos'!$C$34</f>
         <v/>
       </c>
-      <c r="D60" s="23">
+      <c r="D60" s="24">
         <f>'Supuestos'!$C$34</f>
         <v/>
       </c>
@@ -5689,6 +5964,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I60" s="18">
+        <f>IF(AND(ISNUMBER(C60),C60&gt;=0,C60&lt;=1),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="B61" t="inlineStr">
@@ -5696,15 +5975,15 @@
           <t>Comisiones (pasarela + ventas)</t>
         </is>
       </c>
-      <c r="E61" s="19">
+      <c r="E61" s="20">
         <f>$E$57*($C$59+$C$60)</f>
         <v/>
       </c>
-      <c r="F61" s="19">
+      <c r="F61" s="20">
         <f>'Modelo'!$C$37</f>
         <v/>
       </c>
-      <c r="G61" s="19">
+      <c r="G61" s="20">
         <f>IF(AND(ISNUMBER(E61),ISNUMBER(F61)),E61-F61,"")</f>
         <v/>
       </c>
@@ -5720,11 +5999,11 @@
           <t>Reembolsos y contracargos</t>
         </is>
       </c>
-      <c r="C62" s="22">
+      <c r="C62" s="23">
         <f>'Supuestos'!$C$35</f>
         <v/>
       </c>
-      <c r="D62" s="23">
+      <c r="D62" s="24">
         <f>'Supuestos'!$C$35</f>
         <v/>
       </c>
@@ -5737,6 +6016,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I62" s="18">
+        <f>IF(AND(ISNUMBER(C62),C62&gt;=0,C62&lt;=1),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="B63" t="inlineStr">
@@ -5744,15 +6027,15 @@
           <t>Reembolsos</t>
         </is>
       </c>
-      <c r="E63" s="19">
+      <c r="E63" s="20">
         <f>$E$57*$C$62</f>
         <v/>
       </c>
-      <c r="F63" s="19">
+      <c r="F63" s="20">
         <f>'Modelo'!$C$38</f>
         <v/>
       </c>
-      <c r="G63" s="19">
+      <c r="G63" s="20">
         <f>IF(AND(ISNUMBER(E63),ISNUMBER(F63)),E63-F63,"")</f>
         <v/>
       </c>
@@ -5772,11 +6055,11 @@
         <f>$E$57*(1-$C$59-$C$60-$C$62)</f>
         <v/>
       </c>
-      <c r="F64" s="19">
+      <c r="F64" s="20">
         <f>'Modelo'!$C$39</f>
         <v/>
       </c>
-      <c r="G64" s="19">
+      <c r="G64" s="20">
         <f>IF(AND(ISNUMBER(E64),ISNUMBER(F64)),E64-F64,"")</f>
         <v/>
       </c>
@@ -5809,6 +6092,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I65" s="18">
+        <f>IF(AND(ISNUMBER(C65),C65&gt;=0),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="B66" t="inlineStr">
@@ -5816,15 +6103,15 @@
           <t>Costos por visita (herramientas, WhatsApp, IA)</t>
         </is>
       </c>
-      <c r="E66" s="19">
+      <c r="E66" s="20">
         <f>$E$10*$C$65</f>
         <v/>
       </c>
-      <c r="F66" s="19">
+      <c r="F66" s="20">
         <f>'Modelo'!$C$40</f>
         <v/>
       </c>
-      <c r="G66" s="19">
+      <c r="G66" s="20">
         <f>IF(AND(ISNUMBER(E66),ISNUMBER(F66)),E66-F66,"")</f>
         <v/>
       </c>
@@ -5840,11 +6127,11 @@
           <t>Costos fijos por mes</t>
         </is>
       </c>
-      <c r="C67" s="18">
+      <c r="C67" s="19">
         <f>'Supuestos'!$C$37</f>
         <v/>
       </c>
-      <c r="D67" s="19">
+      <c r="D67" s="20">
         <f>'Supuestos'!$C$37</f>
         <v/>
       </c>
@@ -5857,6 +6144,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I67" s="18">
+        <f>IF(AND(ISNUMBER(C67),C67&gt;=0),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="B68" s="4" t="inlineStr">
@@ -5868,11 +6159,11 @@
         <f>$E$64-$E$66-$C$67-$C$9</f>
         <v/>
       </c>
-      <c r="F68" s="19">
+      <c r="F68" s="20">
         <f>'Modelo'!$C$41</f>
         <v/>
       </c>
-      <c r="G68" s="19">
+      <c r="G68" s="20">
         <f>IF(AND(ISNUMBER(E68),ISNUMBER(F68)),E68-F68,"")</f>
         <v/>
       </c>
@@ -5888,15 +6179,15 @@
           <t>ROAS sobre facturado</t>
         </is>
       </c>
-      <c r="E69" s="26">
+      <c r="E69" s="27">
         <f>IF($C$9=0,0,$E$48/$C$9)</f>
         <v/>
       </c>
-      <c r="F69" s="26">
+      <c r="F69" s="27">
         <f>'Modelo'!$C$42</f>
         <v/>
       </c>
-      <c r="G69" s="26">
+      <c r="G69" s="27">
         <f>IF(AND(ISNUMBER(E69),ISNUMBER(F69)),E69-F69,"")</f>
         <v/>
       </c>
@@ -5916,11 +6207,11 @@
         <f>IF($C$9=0,0,$E$64/$C$9)</f>
         <v/>
       </c>
-      <c r="F70" s="26">
+      <c r="F70" s="27">
         <f>'Modelo'!$C$43</f>
         <v/>
       </c>
-      <c r="G70" s="26">
+      <c r="G70" s="27">
         <f>IF(AND(ISNUMBER(E70),ISNUMBER(F70)),E70-F70,"")</f>
         <v/>
       </c>
@@ -5936,15 +6227,15 @@
           <t>Margen sobre cash</t>
         </is>
       </c>
-      <c r="E71" s="23">
+      <c r="E71" s="24">
         <f>IF($E$57=0,0,$E$68/$E$57)</f>
         <v/>
       </c>
-      <c r="F71" s="23">
+      <c r="F71" s="24">
         <f>'Modelo'!$C$44</f>
         <v/>
       </c>
-      <c r="G71" s="23">
+      <c r="G71" s="24">
         <f>IF(AND(ISNUMBER(E71),ISNUMBER(F71)),E71-F71,"")</f>
         <v/>
       </c>
@@ -5960,11 +6251,11 @@
           <t>ROAS objetivo sobre cash neto</t>
         </is>
       </c>
-      <c r="C72" s="27">
+      <c r="C72" s="28">
         <f>'Supuestos'!$C$45</f>
         <v/>
       </c>
-      <c r="D72" s="26">
+      <c r="D72" s="27">
         <f>'Supuestos'!$C$45</f>
         <v/>
       </c>
@@ -5977,6 +6268,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I72" s="18">
+        <f>IF(AND(ISNUMBER(C72),C72&gt;=0),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="B73" t="inlineStr">
@@ -5984,11 +6279,11 @@
           <t>¿Cumple el ROAS objetivo?</t>
         </is>
       </c>
-      <c r="E73" s="28">
+      <c r="E73" s="29">
         <f>IF($E$70&gt;=$C$72,"SÍ","NO")</f>
         <v/>
       </c>
-      <c r="F73" s="28">
+      <c r="F73" s="29">
         <f>'Modelo'!$C$45</f>
         <v/>
       </c>
@@ -6069,11 +6364,11 @@
           <t>Margen de seguridad</t>
         </is>
       </c>
-      <c r="C77" s="22">
+      <c r="C77" s="23">
         <f>'Supuestos'!$C$46</f>
         <v/>
       </c>
-      <c r="D77" s="23">
+      <c r="D77" s="24">
         <f>'Supuestos'!$C$46</f>
         <v/>
       </c>
@@ -6085,6 +6380,10 @@
         <is>
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
+      </c>
+      <c r="I77" s="18">
+        <f>IF(AND(ISNUMBER(C77),C77&gt;=0,C77&lt;=1),"OK","REVISAR")</f>
+        <v/>
       </c>
     </row>
     <row r="78">
@@ -6254,7 +6553,7 @@
         <f>IF($E$8&gt;$E$76,"ROJO",IF(AND($E$8&lt;=$E$78,$E$70&gt;=$C$72),"VERDE","AMARILLO"))</f>
         <v/>
       </c>
-      <c r="F85" s="28">
+      <c r="F85" s="29">
         <f>'Modelo'!$C$56</f>
         <v/>
       </c>
@@ -6274,11 +6573,11 @@
           <t>Meta de ventas del producto principal</t>
         </is>
       </c>
-      <c r="C86" s="29">
+      <c r="C86" s="30">
         <f>'Supuestos'!$C$47</f>
         <v/>
       </c>
-      <c r="D86" s="21">
+      <c r="D86" s="22">
         <f>'Supuestos'!$C$47</f>
         <v/>
       </c>
@@ -6291,6 +6590,10 @@
           <t>Supuesto. Escribí encima para probar; la base queda al lado.</t>
         </is>
       </c>
+      <c r="I86" s="18">
+        <f>IF(AND(ISNUMBER(C86),C86&gt;=0),"OK","REVISAR")</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="B87" s="4" t="inlineStr">
@@ -6302,11 +6605,11 @@
         <f>IF($E$15=0,"inalcanzable con estos supuestos",$C$86/$E$15*$E$8)</f>
         <v/>
       </c>
-      <c r="F87" s="19">
+      <c r="F87" s="20">
         <f>'Modelo'!$C$57</f>
         <v/>
       </c>
-      <c r="G87" s="19">
+      <c r="G87" s="20">
         <f>IF(AND(ISNUMBER(E87),ISNUMBER(F87)),E87-F87,"")</f>
         <v/>
       </c>
@@ -6322,15 +6625,15 @@
           <t>Inversión para la meta al costo objetivo (lo máximo que conviene pagar)</t>
         </is>
       </c>
-      <c r="E88" s="19">
+      <c r="E88" s="20">
         <f>IF($E$15=0,"inalcanzable con estos supuestos",$C$86/$E$15*$E$78)</f>
         <v/>
       </c>
-      <c r="F88" s="19">
+      <c r="F88" s="20">
         <f>'Modelo'!$C$58</f>
         <v/>
       </c>
-      <c r="G88" s="19">
+      <c r="G88" s="20">
         <f>IF(AND(ISNUMBER(E88),ISNUMBER(F88)),E88-F88,"")</f>
         <v/>
       </c>
@@ -6470,39 +6773,61 @@
         </is>
       </c>
     </row>
+    <row r="98" ht="30" customHeight="1">
+      <c r="B98" s="5" t="inlineStr">
+        <is>
+          <t>La columna Rango avisa si escribiste algo imposible (un porcentaje fuera de 0 a 1, un negativo, texto) y Chequeos repite los chequeos del modelo con tus números del Simulador.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="B97:H97"/>
+    <mergeCell ref="B98:H98"/>
     <mergeCell ref="B95:H95"/>
     <mergeCell ref="B96:H96"/>
   </mergeCells>
+  <conditionalFormatting sqref="I6:I93">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
+      <formula>"REVISAR"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C6:C93">
-    <cfRule type="expression" priority="1" dxfId="3">
+    <cfRule type="expression" priority="2" dxfId="3">
       <formula>AND(ISNUMBER(C6),C6&lt;&gt;D6)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E73:F73">
-    <cfRule type="expression" priority="2" dxfId="0">
+    <cfRule type="expression" priority="3" dxfId="0">
       <formula>LEFT(E73,5)="VERDE"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="1">
+    <cfRule type="expression" priority="4" dxfId="1">
       <formula>LEFT(E73,8)="AMARILLO"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="2">
+    <cfRule type="expression" priority="5" dxfId="2">
       <formula>LEFT(E73,4)="ROJO"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E85:F85">
-    <cfRule type="expression" priority="5" dxfId="0">
+    <cfRule type="expression" priority="6" dxfId="0">
       <formula>LEFT(E85,5)="VERDE"</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="1">
+    <cfRule type="expression" priority="7" dxfId="1">
       <formula>LEFT(E85,8)="AMARILLO"</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" dxfId="2">
+    <cfRule type="expression" priority="8" dxfId="2">
       <formula>LEFT(E85,4)="ROJO"</formula>
     </cfRule>
   </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="C11 C13 C20 C24 C28 C32 C36 C40 C44 C54 C55 C56 C59 C60 C62 C77" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Porcentaje fuera de rango" error="Escribí el porcentaje como fracción entre 0 y 1 (15 % = 0,15)." type="decimal" operator="between">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation sqref="C7 C9 C18 C22 C26 C30 C34 C38 C42 C46 C65 C67 C72 C86" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Valor inválido" error="Tiene que ser un número mayor o igual a 0." type="decimal" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>
     <oddHeader>&amp;CJesús Tassarolo · TooAudience&amp;R&amp;D</oddHeader>
@@ -6604,7 +6929,7 @@
           <t>Visitas a la página de ventas (VSL)</t>
         </is>
       </c>
-      <c r="C6" s="21">
+      <c r="C6" s="22">
         <f>'Modelo'!$C$8</f>
         <v/>
       </c>
@@ -6613,7 +6938,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E6" s="25">
+      <c r="E6" s="26">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$8/'Modelo'!$C$8)</f>
         <v/>
       </c>
@@ -6641,15 +6966,15 @@
           <t>Abren el checkout</t>
         </is>
       </c>
-      <c r="C7" s="21">
+      <c r="C7" s="22">
         <f>'Modelo'!$C$9</f>
         <v/>
       </c>
-      <c r="D7" s="23">
+      <c r="D7" s="24">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$9/'Modelo'!$C$8)</f>
         <v/>
       </c>
-      <c r="E7" s="25">
+      <c r="E7" s="26">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$9/'Modelo'!$C$8)</f>
         <v/>
       </c>
@@ -6677,15 +7002,15 @@
           <t>Compran el producto principal</t>
         </is>
       </c>
-      <c r="C8" s="21">
+      <c r="C8" s="22">
         <f>'Modelo'!$C$10</f>
         <v/>
       </c>
-      <c r="D8" s="23">
+      <c r="D8" s="24">
         <f>IF('Modelo'!$C$9=0,0,'Modelo'!$C$10/'Modelo'!$C$9)</f>
         <v/>
       </c>
-      <c r="E8" s="25">
+      <c r="E8" s="26">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$10/'Modelo'!$C$8)</f>
         <v/>
       </c>
@@ -6713,15 +7038,15 @@
           <t>Toman el bump 1</t>
         </is>
       </c>
-      <c r="C9" s="21">
+      <c r="C9" s="22">
         <f>'Modelo'!$C$15</f>
         <v/>
       </c>
-      <c r="D9" s="23">
+      <c r="D9" s="24">
         <f>IF('Modelo'!$C$10=0,0,'Modelo'!$C$15/'Modelo'!$C$10)</f>
         <v/>
       </c>
-      <c r="E9" s="25">
+      <c r="E9" s="26">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$15/'Modelo'!$C$8)</f>
         <v/>
       </c>
@@ -6752,15 +7077,15 @@
           <t>Toman el bump 2</t>
         </is>
       </c>
-      <c r="C10" s="21">
+      <c r="C10" s="22">
         <f>'Modelo'!$C$17</f>
         <v/>
       </c>
-      <c r="D10" s="23">
+      <c r="D10" s="24">
         <f>IF('Modelo'!$C$10=0,0,'Modelo'!$C$17/'Modelo'!$C$10)</f>
         <v/>
       </c>
-      <c r="E10" s="25">
+      <c r="E10" s="26">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$17/'Modelo'!$C$8)</f>
         <v/>
       </c>
@@ -6791,15 +7116,15 @@
           <t>Toman la OTO 1</t>
         </is>
       </c>
-      <c r="C11" s="21">
+      <c r="C11" s="22">
         <f>'Modelo'!$C$19</f>
         <v/>
       </c>
-      <c r="D11" s="23">
+      <c r="D11" s="24">
         <f>IF('Modelo'!$C$10=0,0,'Modelo'!$C$19/'Modelo'!$C$10)</f>
         <v/>
       </c>
-      <c r="E11" s="25">
+      <c r="E11" s="26">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$19/'Modelo'!$C$8)</f>
         <v/>
       </c>
@@ -6830,15 +7155,15 @@
           <t>Toman la OTO 2</t>
         </is>
       </c>
-      <c r="C12" s="21">
+      <c r="C12" s="22">
         <f>'Modelo'!$C$21</f>
         <v/>
       </c>
-      <c r="D12" s="23">
+      <c r="D12" s="24">
         <f>IF('Modelo'!$C$10=0,0,'Modelo'!$C$21/'Modelo'!$C$10)</f>
         <v/>
       </c>
-      <c r="E12" s="25">
+      <c r="E12" s="26">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$21/'Modelo'!$C$8)</f>
         <v/>
       </c>
@@ -6869,15 +7194,15 @@
           <t>Toman la OTO 3</t>
         </is>
       </c>
-      <c r="C13" s="21">
+      <c r="C13" s="22">
         <f>'Modelo'!$C$23</f>
         <v/>
       </c>
-      <c r="D13" s="23">
+      <c r="D13" s="24">
         <f>IF('Modelo'!$C$10=0,0,'Modelo'!$C$23/'Modelo'!$C$10)</f>
         <v/>
       </c>
-      <c r="E13" s="25">
+      <c r="E13" s="26">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$23/'Modelo'!$C$8)</f>
         <v/>
       </c>
@@ -6908,15 +7233,15 @@
           <t>Toman la OTO 4</t>
         </is>
       </c>
-      <c r="C14" s="21">
+      <c r="C14" s="22">
         <f>'Modelo'!$C$25</f>
         <v/>
       </c>
-      <c r="D14" s="23">
+      <c r="D14" s="24">
         <f>IF('Modelo'!$C$10=0,0,'Modelo'!$C$25/'Modelo'!$C$10)</f>
         <v/>
       </c>
-      <c r="E14" s="25">
+      <c r="E14" s="26">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$25/'Modelo'!$C$8)</f>
         <v/>
       </c>
@@ -6947,15 +7272,15 @@
           <t>Ascienden al programa</t>
         </is>
       </c>
-      <c r="C15" s="21">
+      <c r="C15" s="22">
         <f>'Modelo'!$C$27</f>
         <v/>
       </c>
-      <c r="D15" s="23">
+      <c r="D15" s="24">
         <f>IF('Modelo'!$C$10=0,0,'Modelo'!$C$27/'Modelo'!$C$10)</f>
         <v/>
       </c>
-      <c r="E15" s="25">
+      <c r="E15" s="26">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$27/'Modelo'!$C$8)</f>
         <v/>
       </c>
@@ -7157,7 +7482,7 @@
           <t>Escenario en uso (1 = conservador · 2 = base · 3 = optimista)</t>
         </is>
       </c>
-      <c r="C6" s="29" t="n">
+      <c r="C6" s="30" t="n">
         <v>2</v>
       </c>
       <c r="G6" t="inlineStr">
@@ -7190,7 +7515,7 @@
           <t>Inversión en publicidad por mes</t>
         </is>
       </c>
-      <c r="C8" s="18" t="n">
+      <c r="C8" s="19" t="n">
         <v>9000</v>
       </c>
       <c r="G8" t="inlineStr">
@@ -7253,17 +7578,17 @@
           <t>% de visitas que llegan al checkout</t>
         </is>
       </c>
-      <c r="C12" s="23">
+      <c r="C12" s="24">
         <f>IF('Supuestos'!$C$6=1,D12,IF('Supuestos'!$C$6=2,E12,F12))</f>
         <v/>
       </c>
-      <c r="D12" s="22" t="n">
+      <c r="D12" s="23" t="n">
         <v>0.025</v>
       </c>
-      <c r="E12" s="22" t="n">
+      <c r="E12" s="23" t="n">
         <v>0.035</v>
       </c>
-      <c r="F12" s="22" t="n">
+      <c r="F12" s="23" t="n">
         <v>0.045</v>
       </c>
       <c r="G12" t="inlineStr">
@@ -7283,17 +7608,17 @@
           <t>% de checkouts que terminan en compra</t>
         </is>
       </c>
-      <c r="C13" s="23">
+      <c r="C13" s="24">
         <f>IF('Supuestos'!$C$6=1,D13,IF('Supuestos'!$C$6=2,E13,F13))</f>
         <v/>
       </c>
-      <c r="D13" s="22" t="n">
+      <c r="D13" s="23" t="n">
         <v>0.2</v>
       </c>
-      <c r="E13" s="22" t="n">
+      <c r="E13" s="23" t="n">
         <v>0.26</v>
       </c>
-      <c r="F13" s="22" t="n">
+      <c r="F13" s="23" t="n">
         <v>0.3</v>
       </c>
       <c r="G13" t="inlineStr">
@@ -7366,17 +7691,17 @@
           <t>Bump 1: % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C18" s="23">
+      <c r="C18" s="24">
         <f>IF('Supuestos'!$C$6=1,D18,IF('Supuestos'!$C$6=2,E18,F18))</f>
         <v/>
       </c>
-      <c r="D18" s="22" t="n">
+      <c r="D18" s="23" t="n">
         <v>0.18</v>
       </c>
-      <c r="E18" s="22" t="n">
+      <c r="E18" s="23" t="n">
         <v>0.25</v>
       </c>
-      <c r="F18" s="22" t="n">
+      <c r="F18" s="23" t="n">
         <v>0.35</v>
       </c>
       <c r="G18" t="inlineStr">
@@ -7412,17 +7737,17 @@
           <t>Bump 2: % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C20" s="23">
+      <c r="C20" s="24">
         <f>IF('Supuestos'!$C$6=1,D20,IF('Supuestos'!$C$6=2,E20,F20))</f>
         <v/>
       </c>
-      <c r="D20" s="22" t="n">
+      <c r="D20" s="23" t="n">
         <v>0.12</v>
       </c>
-      <c r="E20" s="22" t="n">
+      <c r="E20" s="23" t="n">
         <v>0.18</v>
       </c>
-      <c r="F20" s="22" t="n">
+      <c r="F20" s="23" t="n">
         <v>0.25</v>
       </c>
       <c r="G20" t="inlineStr">
@@ -7458,17 +7783,17 @@
           <t>OTO 1: % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C22" s="23">
+      <c r="C22" s="24">
         <f>IF('Supuestos'!$C$6=1,D22,IF('Supuestos'!$C$6=2,E22,F22))</f>
         <v/>
       </c>
-      <c r="D22" s="22" t="n">
+      <c r="D22" s="23" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="E22" s="22" t="n">
+      <c r="E22" s="23" t="n">
         <v>0.1</v>
       </c>
-      <c r="F22" s="22" t="n">
+      <c r="F22" s="23" t="n">
         <v>0.14</v>
       </c>
       <c r="G22" t="inlineStr">
@@ -7504,17 +7829,17 @@
           <t>OTO 2: % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C24" s="23">
+      <c r="C24" s="24">
         <f>IF('Supuestos'!$C$6=1,D24,IF('Supuestos'!$C$6=2,E24,F24))</f>
         <v/>
       </c>
-      <c r="D24" s="22" t="n">
+      <c r="D24" s="23" t="n">
         <v>0.04</v>
       </c>
-      <c r="E24" s="22" t="n">
+      <c r="E24" s="23" t="n">
         <v>0.06</v>
       </c>
-      <c r="F24" s="22" t="n">
+      <c r="F24" s="23" t="n">
         <v>0.09</v>
       </c>
       <c r="G24" t="inlineStr">
@@ -7550,17 +7875,17 @@
           <t>OTO 3: % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C26" s="23">
+      <c r="C26" s="24">
         <f>IF('Supuestos'!$C$6=1,D26,IF('Supuestos'!$C$6=2,E26,F26))</f>
         <v/>
       </c>
-      <c r="D26" s="22" t="n">
+      <c r="D26" s="23" t="n">
         <v>0.02</v>
       </c>
-      <c r="E26" s="22" t="n">
+      <c r="E26" s="23" t="n">
         <v>0.03</v>
       </c>
-      <c r="F26" s="22" t="n">
+      <c r="F26" s="23" t="n">
         <v>0.05</v>
       </c>
       <c r="G26" t="inlineStr">
@@ -7596,17 +7921,17 @@
           <t>OTO 4: % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C28" s="23">
+      <c r="C28" s="24">
         <f>IF('Supuestos'!$C$6=1,D28,IF('Supuestos'!$C$6=2,E28,F28))</f>
         <v/>
       </c>
-      <c r="D28" s="22" t="n">
+      <c r="D28" s="23" t="n">
         <v>0.03</v>
       </c>
-      <c r="E28" s="22" t="n">
+      <c r="E28" s="23" t="n">
         <v>0.04</v>
       </c>
-      <c r="F28" s="22" t="n">
+      <c r="F28" s="23" t="n">
         <v>0.06</v>
       </c>
       <c r="G28" t="inlineStr">
@@ -7642,17 +7967,17 @@
           <t>Ascensión (programa de mayor valor): % de compradores que lo toman</t>
         </is>
       </c>
-      <c r="C30" s="23">
+      <c r="C30" s="24">
         <f>IF('Supuestos'!$C$6=1,D30,IF('Supuestos'!$C$6=2,E30,F30))</f>
         <v/>
       </c>
-      <c r="D30" s="22" t="n">
+      <c r="D30" s="23" t="n">
         <v>0.01</v>
       </c>
-      <c r="E30" s="22" t="n">
+      <c r="E30" s="23" t="n">
         <v>0.02</v>
       </c>
-      <c r="F30" s="22" t="n">
+      <c r="F30" s="23" t="n">
         <v>0.04</v>
       </c>
       <c r="G30" t="inlineStr">
@@ -7681,7 +8006,7 @@
           <t>Comisión de la pasarela o plataforma de pago</t>
         </is>
       </c>
-      <c r="C33" s="22" t="n">
+      <c r="C33" s="23" t="n">
         <v>0.1</v>
       </c>
       <c r="G33" t="inlineStr">
@@ -7701,7 +8026,7 @@
           <t>Comisión del equipo de ventas</t>
         </is>
       </c>
-      <c r="C34" s="22" t="n">
+      <c r="C34" s="23" t="n">
         <v>0</v>
       </c>
       <c r="G34" t="inlineStr">
@@ -7721,7 +8046,7 @@
           <t>Reembolsos y contracargos</t>
         </is>
       </c>
-      <c r="C35" s="22" t="n">
+      <c r="C35" s="23" t="n">
         <v>0.05</v>
       </c>
       <c r="G35" t="inlineStr">
@@ -7761,7 +8086,7 @@
           <t>Costos fijos por mes</t>
         </is>
       </c>
-      <c r="C37" s="18" t="n">
+      <c r="C37" s="19" t="n">
         <v>1500</v>
       </c>
       <c r="G37" t="inlineStr">
@@ -7794,7 +8119,7 @@
           <t>% del facturado que entra en el mes 1</t>
         </is>
       </c>
-      <c r="C40" s="22" t="n">
+      <c r="C40" s="23" t="n">
         <v>1</v>
       </c>
       <c r="G40" t="inlineStr">
@@ -7814,7 +8139,7 @@
           <t>% que entra en el mes 2</t>
         </is>
       </c>
-      <c r="C41" s="22" t="n">
+      <c r="C41" s="23" t="n">
         <v>0</v>
       </c>
       <c r="G41" t="inlineStr">
@@ -7834,7 +8159,7 @@
           <t>% que entra en el mes 3</t>
         </is>
       </c>
-      <c r="C42" s="22" t="n">
+      <c r="C42" s="23" t="n">
         <v>0</v>
       </c>
       <c r="G42" t="inlineStr">
@@ -7867,7 +8192,7 @@
           <t>ROAS objetivo sobre cash neto</t>
         </is>
       </c>
-      <c r="C45" s="27" t="n">
+      <c r="C45" s="28" t="n">
         <v>2</v>
       </c>
       <c r="G45" t="inlineStr">
@@ -7887,7 +8212,7 @@
           <t>Margen de seguridad</t>
         </is>
       </c>
-      <c r="C46" s="22" t="n">
+      <c r="C46" s="23" t="n">
         <v>0.3</v>
       </c>
       <c r="G46" t="inlineStr">
@@ -7907,7 +8232,7 @@
           <t>Meta de ventas del producto principal</t>
         </is>
       </c>
-      <c r="C47" s="29" t="n">
+      <c r="C47" s="30" t="n">
         <v>500</v>
       </c>
       <c r="G47" t="inlineStr">
@@ -7927,7 +8252,7 @@
           <t>Crecimiento de la inversión por mes (proyección)</t>
         </is>
       </c>
-      <c r="C48" s="22" t="n">
+      <c r="C48" s="23" t="n">
         <v>0.1</v>
       </c>
       <c r="G48" t="inlineStr">
@@ -7947,7 +8272,7 @@
           <t>Caja inicial</t>
         </is>
       </c>
-      <c r="C49" s="18" t="n">
+      <c r="C49" s="19" t="n">
         <v>5000</v>
       </c>
       <c r="G49" t="inlineStr">
@@ -8058,7 +8383,7 @@
           <t>Visitas a la página de ventas</t>
         </is>
       </c>
-      <c r="C8" s="20">
+      <c r="C8" s="21">
         <f>IF('Modelo'!$C$7=0,0,'Supuestos'!$C$8/'Modelo'!$C$7)</f>
         <v/>
       </c>
@@ -8074,7 +8399,7 @@
           <t>Checkouts iniciados</t>
         </is>
       </c>
-      <c r="C9" s="21">
+      <c r="C9" s="22">
         <f>'Modelo'!$C$8*'Supuestos'!$C$12</f>
         <v/>
       </c>
@@ -8106,7 +8431,7 @@
           <t>% de visitas que compran</t>
         </is>
       </c>
-      <c r="C11" s="25">
+      <c r="C11" s="26">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$10/'Modelo'!$C$8)</f>
         <v/>
       </c>
@@ -8147,7 +8472,7 @@
           <t>Facturado: producto principal</t>
         </is>
       </c>
-      <c r="C14" s="19">
+      <c r="C14" s="20">
         <f>'Modelo'!$C$10*'Supuestos'!$C$16</f>
         <v/>
       </c>
@@ -8163,7 +8488,7 @@
           <t>Ventas: Bump 1</t>
         </is>
       </c>
-      <c r="C15" s="24">
+      <c r="C15" s="25">
         <f>'Modelo'!$C$10*'Supuestos'!$C$18</f>
         <v/>
       </c>
@@ -8179,7 +8504,7 @@
           <t>Facturado: Bump 1</t>
         </is>
       </c>
-      <c r="C16" s="19">
+      <c r="C16" s="20">
         <f>'Modelo'!$C$15*'Supuestos'!$C$17</f>
         <v/>
       </c>
@@ -8195,7 +8520,7 @@
           <t>Ventas: Bump 2</t>
         </is>
       </c>
-      <c r="C17" s="24">
+      <c r="C17" s="25">
         <f>'Modelo'!$C$10*'Supuestos'!$C$20</f>
         <v/>
       </c>
@@ -8211,7 +8536,7 @@
           <t>Facturado: Bump 2</t>
         </is>
       </c>
-      <c r="C18" s="19">
+      <c r="C18" s="20">
         <f>'Modelo'!$C$17*'Supuestos'!$C$19</f>
         <v/>
       </c>
@@ -8227,7 +8552,7 @@
           <t>Ventas: OTO 1</t>
         </is>
       </c>
-      <c r="C19" s="24">
+      <c r="C19" s="25">
         <f>'Modelo'!$C$10*'Supuestos'!$C$22</f>
         <v/>
       </c>
@@ -8243,7 +8568,7 @@
           <t>Facturado: OTO 1</t>
         </is>
       </c>
-      <c r="C20" s="19">
+      <c r="C20" s="20">
         <f>'Modelo'!$C$19*'Supuestos'!$C$21</f>
         <v/>
       </c>
@@ -8259,7 +8584,7 @@
           <t>Ventas: OTO 2</t>
         </is>
       </c>
-      <c r="C21" s="24">
+      <c r="C21" s="25">
         <f>'Modelo'!$C$10*'Supuestos'!$C$24</f>
         <v/>
       </c>
@@ -8275,7 +8600,7 @@
           <t>Facturado: OTO 2</t>
         </is>
       </c>
-      <c r="C22" s="19">
+      <c r="C22" s="20">
         <f>'Modelo'!$C$21*'Supuestos'!$C$23</f>
         <v/>
       </c>
@@ -8291,7 +8616,7 @@
           <t>Ventas: OTO 3</t>
         </is>
       </c>
-      <c r="C23" s="24">
+      <c r="C23" s="25">
         <f>'Modelo'!$C$10*'Supuestos'!$C$26</f>
         <v/>
       </c>
@@ -8307,7 +8632,7 @@
           <t>Facturado: OTO 3</t>
         </is>
       </c>
-      <c r="C24" s="19">
+      <c r="C24" s="20">
         <f>'Modelo'!$C$23*'Supuestos'!$C$25</f>
         <v/>
       </c>
@@ -8323,7 +8648,7 @@
           <t>Ventas: OTO 4</t>
         </is>
       </c>
-      <c r="C25" s="24">
+      <c r="C25" s="25">
         <f>'Modelo'!$C$10*'Supuestos'!$C$28</f>
         <v/>
       </c>
@@ -8339,7 +8664,7 @@
           <t>Facturado: OTO 4</t>
         </is>
       </c>
-      <c r="C26" s="19">
+      <c r="C26" s="20">
         <f>'Modelo'!$C$25*'Supuestos'!$C$27</f>
         <v/>
       </c>
@@ -8355,7 +8680,7 @@
           <t>Ventas: Ascensión (programa de mayor valor)</t>
         </is>
       </c>
-      <c r="C27" s="24">
+      <c r="C27" s="25">
         <f>'Modelo'!$C$10*'Supuestos'!$C$30</f>
         <v/>
       </c>
@@ -8371,7 +8696,7 @@
           <t>Facturado: Ascensión (programa de mayor valor)</t>
         </is>
       </c>
-      <c r="C28" s="19">
+      <c r="C28" s="20">
         <f>'Modelo'!$C$27*'Supuestos'!$C$29</f>
         <v/>
       </c>
@@ -8419,7 +8744,7 @@
           <t>AOV ÷ precio del principal</t>
         </is>
       </c>
-      <c r="C31" s="26">
+      <c r="C31" s="27">
         <f>IF('Supuestos'!$C$16=0,0,'Modelo'!$C$30/'Supuestos'!$C$16)</f>
         <v/>
       </c>
@@ -8435,7 +8760,7 @@
           <t>Ventas del principal por visita (para la proyección)</t>
         </is>
       </c>
-      <c r="C32" s="25">
+      <c r="C32" s="26">
         <f>IF('Modelo'!$C$8=0,0,'Modelo'!$C$10/'Modelo'!$C$8)</f>
         <v/>
       </c>
@@ -8476,7 +8801,7 @@
           <t>Cash a cobrar (facturado × cobranza completa)</t>
         </is>
       </c>
-      <c r="C35" s="19">
+      <c r="C35" s="20">
         <f>'Modelo'!$C$29*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42)</f>
         <v/>
       </c>
@@ -8492,7 +8817,7 @@
           <t>Cash que entra en el primer mes</t>
         </is>
       </c>
-      <c r="C36" s="19">
+      <c r="C36" s="20">
         <f>'Modelo'!$C$29*'Supuestos'!$C$40</f>
         <v/>
       </c>
@@ -8508,7 +8833,7 @@
           <t>Comisiones (pasarela + ventas)</t>
         </is>
       </c>
-      <c r="C37" s="19">
+      <c r="C37" s="20">
         <f>'Modelo'!$C$35*('Supuestos'!$C$33+'Supuestos'!$C$34)</f>
         <v/>
       </c>
@@ -8524,7 +8849,7 @@
           <t>Reembolsos</t>
         </is>
       </c>
-      <c r="C38" s="19">
+      <c r="C38" s="20">
         <f>'Modelo'!$C$35*'Supuestos'!$C$35</f>
         <v/>
       </c>
@@ -8556,7 +8881,7 @@
           <t>Costos por visita (herramientas, WhatsApp, IA)</t>
         </is>
       </c>
-      <c r="C40" s="19">
+      <c r="C40" s="20">
         <f>'Modelo'!$C$8*'Supuestos'!$C$36</f>
         <v/>
       </c>
@@ -8588,7 +8913,7 @@
           <t>ROAS sobre facturado</t>
         </is>
       </c>
-      <c r="C42" s="26">
+      <c r="C42" s="27">
         <f>IF('Supuestos'!$C$8=0,0,'Modelo'!$C$29/'Supuestos'!$C$8)</f>
         <v/>
       </c>
@@ -8620,7 +8945,7 @@
           <t>Margen sobre cash</t>
         </is>
       </c>
-      <c r="C44" s="23">
+      <c r="C44" s="24">
         <f>IF('Modelo'!$C$35=0,0,'Modelo'!$C$41/'Modelo'!$C$35)</f>
         <v/>
       </c>
@@ -8636,7 +8961,7 @@
           <t>¿Cumple el ROAS objetivo?</t>
         </is>
       </c>
-      <c r="C45" s="28">
+      <c r="C45" s="29">
         <f>IF('Modelo'!$C$43&gt;='Supuestos'!$C$45,"SÍ","NO")</f>
         <v/>
       </c>
@@ -8830,7 +9155,7 @@
           <t>Inversión para la meta al costo objetivo (lo máximo que conviene pagar)</t>
         </is>
       </c>
-      <c r="C58" s="19">
+      <c r="C58" s="20">
         <f>IF('Modelo'!$C$11=0,"inalcanzable con estos supuestos",'Supuestos'!$C$47/'Modelo'!$C$11*'Modelo'!$C$49)</f>
         <v/>
       </c>
@@ -8970,7 +9295,7 @@
           <t>Umbral de 'cerca del cero' (inversión × margen de seguridad)</t>
         </is>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="20">
         <f>'Supuestos'!$C$8*'Supuestos'!$C$46</f>
         <v/>
       </c>
@@ -8995,143 +9320,143 @@
           <t>Precio ↓  /  % checkout → compra →</t>
         </is>
       </c>
-      <c r="C9" s="30" t="n">
+      <c r="C9" s="31" t="n">
         <v>0.18</v>
       </c>
-      <c r="D9" s="30" t="n">
+      <c r="D9" s="31" t="n">
         <v>0.22</v>
       </c>
-      <c r="E9" s="30" t="n">
+      <c r="E9" s="31" t="n">
         <v>0.26</v>
       </c>
-      <c r="F9" s="30" t="n">
+      <c r="F9" s="31" t="n">
         <v>0.3</v>
       </c>
-      <c r="G9" s="30" t="n">
+      <c r="G9" s="31" t="n">
         <v>0.34</v>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="31" t="n">
+      <c r="B10" s="32" t="n">
         <v>27</v>
       </c>
-      <c r="C10" s="19">
+      <c r="C10" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*$B10)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="D10" s="19">
+      <c r="D10" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*$B10)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="E10" s="19">
+      <c r="E10" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*$B10)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="F10" s="19">
+      <c r="F10" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*$B10)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="G10" s="19">
+      <c r="G10" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*$B10)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="31" t="n">
+      <c r="B11" s="32" t="n">
         <v>37</v>
       </c>
-      <c r="C11" s="19">
+      <c r="C11" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*$B11)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="D11" s="19">
+      <c r="D11" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*$B11)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="E11" s="19">
+      <c r="E11" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*$B11)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="F11" s="19">
+      <c r="F11" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*$B11)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="G11" s="19">
+      <c r="G11" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*$B11)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="31" t="n">
+      <c r="B12" s="32" t="n">
         <v>47</v>
       </c>
-      <c r="C12" s="19">
+      <c r="C12" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*$B12)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="D12" s="19">
+      <c r="D12" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*$B12)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="E12" s="19">
+      <c r="E12" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*$B12)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="F12" s="19">
+      <c r="F12" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*$B12)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="G12" s="19">
+      <c r="G12" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*$B12)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="31" t="n">
+      <c r="B13" s="32" t="n">
         <v>67</v>
       </c>
-      <c r="C13" s="19">
+      <c r="C13" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*$B13)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="D13" s="19">
+      <c r="D13" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*$B13)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="E13" s="19">
+      <c r="E13" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*$B13)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="F13" s="19">
+      <c r="F13" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*$B13)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="G13" s="19">
+      <c r="G13" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*$B13)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="31" t="n">
+      <c r="B14" s="32" t="n">
         <v>97</v>
       </c>
-      <c r="C14" s="19">
+      <c r="C14" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*$B14)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*C$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="D14" s="19">
+      <c r="D14" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*$B14)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*D$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="E14" s="19">
+      <c r="E14" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*$B14)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*E$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="F14" s="19">
+      <c r="F14" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*$B14)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*F$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="G14" s="19">
+      <c r="G14" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*$B14)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*G$9)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
@@ -9156,224 +9481,224 @@
           <t>Costo por visita ↓  /  % visita → checkout →</t>
         </is>
       </c>
-      <c r="C19" s="30" t="n">
+      <c r="C19" s="31" t="n">
         <v>0.02</v>
       </c>
-      <c r="D19" s="30" t="n">
+      <c r="D19" s="31" t="n">
         <v>0.025</v>
       </c>
-      <c r="E19" s="30" t="n">
+      <c r="E19" s="31" t="n">
         <v>0.03</v>
       </c>
-      <c r="F19" s="30" t="n">
+      <c r="F19" s="31" t="n">
         <v>0.035</v>
       </c>
-      <c r="G19" s="30" t="n">
+      <c r="G19" s="31" t="n">
         <v>0.04</v>
       </c>
-      <c r="H19" s="30" t="n">
+      <c r="H19" s="31" t="n">
         <v>0.05</v>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="32" t="n">
+      <c r="B20" s="33" t="n">
         <v>0.15</v>
       </c>
-      <c r="C20" s="19">
+      <c r="C20" s="20">
         <f>((((((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B20=0,0,'Supuestos'!$C$8/$B20))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="D20" s="19">
+      <c r="D20" s="20">
         <f>((((((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B20=0,0,'Supuestos'!$C$8/$B20))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="E20" s="19">
+      <c r="E20" s="20">
         <f>((((((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B20=0,0,'Supuestos'!$C$8/$B20))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="F20" s="19">
+      <c r="F20" s="20">
         <f>((((((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B20=0,0,'Supuestos'!$C$8/$B20))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="G20" s="19">
+      <c r="G20" s="20">
         <f>((((((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B20=0,0,'Supuestos'!$C$8/$B20))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="H20" s="19">
+      <c r="H20" s="20">
         <f>((((((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B20=0,0,'Supuestos'!$C$8/$B20))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B20=0,0,'Supuestos'!$C$8/$B20))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="32" t="n">
+      <c r="B21" s="33" t="n">
         <v>0.2</v>
       </c>
-      <c r="C21" s="19">
+      <c r="C21" s="20">
         <f>((((((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B21=0,0,'Supuestos'!$C$8/$B21))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="D21" s="19">
+      <c r="D21" s="20">
         <f>((((((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B21=0,0,'Supuestos'!$C$8/$B21))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="E21" s="19">
+      <c r="E21" s="20">
         <f>((((((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B21=0,0,'Supuestos'!$C$8/$B21))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="F21" s="19">
+      <c r="F21" s="20">
         <f>((((((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B21=0,0,'Supuestos'!$C$8/$B21))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="G21" s="19">
+      <c r="G21" s="20">
         <f>((((((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B21=0,0,'Supuestos'!$C$8/$B21))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="H21" s="19">
+      <c r="H21" s="20">
         <f>((((((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B21=0,0,'Supuestos'!$C$8/$B21))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B21=0,0,'Supuestos'!$C$8/$B21))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="32" t="n">
+      <c r="B22" s="33" t="n">
         <v>0.25</v>
       </c>
-      <c r="C22" s="19">
+      <c r="C22" s="20">
         <f>((((((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B22=0,0,'Supuestos'!$C$8/$B22))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="D22" s="19">
+      <c r="D22" s="20">
         <f>((((((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B22=0,0,'Supuestos'!$C$8/$B22))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="E22" s="19">
+      <c r="E22" s="20">
         <f>((((((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B22=0,0,'Supuestos'!$C$8/$B22))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="F22" s="19">
+      <c r="F22" s="20">
         <f>((((((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B22=0,0,'Supuestos'!$C$8/$B22))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="G22" s="19">
+      <c r="G22" s="20">
         <f>((((((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B22=0,0,'Supuestos'!$C$8/$B22))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="H22" s="19">
+      <c r="H22" s="20">
         <f>((((((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B22=0,0,'Supuestos'!$C$8/$B22))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B22=0,0,'Supuestos'!$C$8/$B22))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="32" t="n">
+      <c r="B23" s="33" t="n">
         <v>0.3</v>
       </c>
-      <c r="C23" s="19">
+      <c r="C23" s="20">
         <f>((((((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B23=0,0,'Supuestos'!$C$8/$B23))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="D23" s="19">
+      <c r="D23" s="20">
         <f>((((((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B23=0,0,'Supuestos'!$C$8/$B23))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="E23" s="19">
+      <c r="E23" s="20">
         <f>((((((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B23=0,0,'Supuestos'!$C$8/$B23))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="F23" s="19">
+      <c r="F23" s="20">
         <f>((((((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B23=0,0,'Supuestos'!$C$8/$B23))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="G23" s="19">
+      <c r="G23" s="20">
         <f>((((((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B23=0,0,'Supuestos'!$C$8/$B23))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="H23" s="19">
+      <c r="H23" s="20">
         <f>((((((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B23=0,0,'Supuestos'!$C$8/$B23))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B23=0,0,'Supuestos'!$C$8/$B23))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="32" t="n">
+      <c r="B24" s="33" t="n">
         <v>0.4</v>
       </c>
-      <c r="C24" s="19">
+      <c r="C24" s="20">
         <f>((((((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B24=0,0,'Supuestos'!$C$8/$B24))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="D24" s="19">
+      <c r="D24" s="20">
         <f>((((((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B24=0,0,'Supuestos'!$C$8/$B24))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="E24" s="19">
+      <c r="E24" s="20">
         <f>((((((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B24=0,0,'Supuestos'!$C$8/$B24))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="F24" s="19">
+      <c r="F24" s="20">
         <f>((((((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B24=0,0,'Supuestos'!$C$8/$B24))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="G24" s="19">
+      <c r="G24" s="20">
         <f>((((((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B24=0,0,'Supuestos'!$C$8/$B24))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="H24" s="19">
+      <c r="H24" s="20">
         <f>((((((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B24=0,0,'Supuestos'!$C$8/$B24))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B24=0,0,'Supuestos'!$C$8/$B24))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="32" t="n">
+      <c r="B25" s="33" t="n">
         <v>0.5</v>
       </c>
-      <c r="C25" s="19">
+      <c r="C25" s="20">
         <f>((((((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B25=0,0,'Supuestos'!$C$8/$B25))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="D25" s="19">
+      <c r="D25" s="20">
         <f>((((((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B25=0,0,'Supuestos'!$C$8/$B25))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="E25" s="19">
+      <c r="E25" s="20">
         <f>((((((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B25=0,0,'Supuestos'!$C$8/$B25))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="F25" s="19">
+      <c r="F25" s="20">
         <f>((((((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B25=0,0,'Supuestos'!$C$8/$B25))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="G25" s="19">
+      <c r="G25" s="20">
         <f>((((((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B25=0,0,'Supuestos'!$C$8/$B25))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="H25" s="19">
+      <c r="H25" s="20">
         <f>((((((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B25=0,0,'Supuestos'!$C$8/$B25))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B25=0,0,'Supuestos'!$C$8/$B25))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="32" t="n">
+      <c r="B26" s="33" t="n">
         <v>0.6</v>
       </c>
-      <c r="C26" s="19">
+      <c r="C26" s="20">
         <f>((((((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*C$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B26=0,0,'Supuestos'!$C$8/$B26))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="D26" s="19">
+      <c r="D26" s="20">
         <f>((((((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*D$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B26=0,0,'Supuestos'!$C$8/$B26))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="E26" s="19">
+      <c r="E26" s="20">
         <f>((((((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*E$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B26=0,0,'Supuestos'!$C$8/$B26))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="F26" s="19">
+      <c r="F26" s="20">
         <f>((((((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*F$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B26=0,0,'Supuestos'!$C$8/$B26))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="G26" s="19">
+      <c r="G26" s="20">
         <f>((((((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*G$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B26=0,0,'Supuestos'!$C$8/$B26))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="H26" s="19">
+      <c r="H26" s="20">
         <f>((((((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF($B26=0,0,'Supuestos'!$C$8/$B26))*H$19)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF($B26=0,0,'Supuestos'!$C$8/$B26))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
@@ -9398,143 +9723,143 @@
           <t>Facturación objetivo ↓ / ROAS objetivo →</t>
         </is>
       </c>
-      <c r="C31" s="33" t="n">
+      <c r="C31" s="34" t="n">
         <v>1.5</v>
       </c>
-      <c r="D31" s="33" t="n">
+      <c r="D31" s="34" t="n">
         <v>2</v>
       </c>
-      <c r="E31" s="33" t="n">
+      <c r="E31" s="34" t="n">
         <v>2.5</v>
       </c>
-      <c r="F31" s="33" t="n">
+      <c r="F31" s="34" t="n">
         <v>3</v>
       </c>
-      <c r="G31" s="33" t="n">
+      <c r="G31" s="34" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="31" t="n">
+      <c r="B32" s="32" t="n">
         <v>10000</v>
       </c>
-      <c r="C32" s="19">
+      <c r="C32" s="20">
         <f>$B32/C$31</f>
         <v/>
       </c>
-      <c r="D32" s="19">
+      <c r="D32" s="20">
         <f>$B32/D$31</f>
         <v/>
       </c>
-      <c r="E32" s="19">
+      <c r="E32" s="20">
         <f>$B32/E$31</f>
         <v/>
       </c>
-      <c r="F32" s="19">
+      <c r="F32" s="20">
         <f>$B32/F$31</f>
         <v/>
       </c>
-      <c r="G32" s="19">
+      <c r="G32" s="20">
         <f>$B32/G$31</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="31" t="n">
+      <c r="B33" s="32" t="n">
         <v>20000</v>
       </c>
-      <c r="C33" s="19">
+      <c r="C33" s="20">
         <f>$B33/C$31</f>
         <v/>
       </c>
-      <c r="D33" s="19">
+      <c r="D33" s="20">
         <f>$B33/D$31</f>
         <v/>
       </c>
-      <c r="E33" s="19">
+      <c r="E33" s="20">
         <f>$B33/E$31</f>
         <v/>
       </c>
-      <c r="F33" s="19">
+      <c r="F33" s="20">
         <f>$B33/F$31</f>
         <v/>
       </c>
-      <c r="G33" s="19">
+      <c r="G33" s="20">
         <f>$B33/G$31</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="31" t="n">
+      <c r="B34" s="32" t="n">
         <v>30000</v>
       </c>
-      <c r="C34" s="19">
+      <c r="C34" s="20">
         <f>$B34/C$31</f>
         <v/>
       </c>
-      <c r="D34" s="19">
+      <c r="D34" s="20">
         <f>$B34/D$31</f>
         <v/>
       </c>
-      <c r="E34" s="19">
+      <c r="E34" s="20">
         <f>$B34/E$31</f>
         <v/>
       </c>
-      <c r="F34" s="19">
+      <c r="F34" s="20">
         <f>$B34/F$31</f>
         <v/>
       </c>
-      <c r="G34" s="19">
+      <c r="G34" s="20">
         <f>$B34/G$31</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="31" t="n">
+      <c r="B35" s="32" t="n">
         <v>50000</v>
       </c>
-      <c r="C35" s="19">
+      <c r="C35" s="20">
         <f>$B35/C$31</f>
         <v/>
       </c>
-      <c r="D35" s="19">
+      <c r="D35" s="20">
         <f>$B35/D$31</f>
         <v/>
       </c>
-      <c r="E35" s="19">
+      <c r="E35" s="20">
         <f>$B35/E$31</f>
         <v/>
       </c>
-      <c r="F35" s="19">
+      <c r="F35" s="20">
         <f>$B35/F$31</f>
         <v/>
       </c>
-      <c r="G35" s="19">
+      <c r="G35" s="20">
         <f>$B35/G$31</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="31" t="n">
+      <c r="B36" s="32" t="n">
         <v>100000</v>
       </c>
-      <c r="C36" s="19">
+      <c r="C36" s="20">
         <f>$B36/C$31</f>
         <v/>
       </c>
-      <c r="D36" s="19">
+      <c r="D36" s="20">
         <f>$B36/D$31</f>
         <v/>
       </c>
-      <c r="E36" s="19">
+      <c r="E36" s="20">
         <f>$B36/E$31</f>
         <v/>
       </c>
-      <c r="F36" s="19">
+      <c r="F36" s="20">
         <f>$B36/F$31</f>
         <v/>
       </c>
-      <c r="G36" s="19">
+      <c r="G36" s="20">
         <f>$B36/G$31</f>
         <v/>
       </c>
@@ -9547,51 +9872,51 @@
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="34">
+      <c r="B38" s="35">
         <f>$B32</f>
         <v/>
       </c>
-      <c r="C38" s="21">
+      <c r="C38" s="22">
         <f>IF('Modelo'!$C$33=0,"inalcanzable",$B32/'Modelo'!$C$33)</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="34">
+      <c r="B39" s="35">
         <f>$B33</f>
         <v/>
       </c>
-      <c r="C39" s="21">
+      <c r="C39" s="22">
         <f>IF('Modelo'!$C$33=0,"inalcanzable",$B33/'Modelo'!$C$33)</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="34">
+      <c r="B40" s="35">
         <f>$B34</f>
         <v/>
       </c>
-      <c r="C40" s="21">
+      <c r="C40" s="22">
         <f>IF('Modelo'!$C$33=0,"inalcanzable",$B34/'Modelo'!$C$33)</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="34">
+      <c r="B41" s="35">
         <f>$B35</f>
         <v/>
       </c>
-      <c r="C41" s="21">
+      <c r="C41" s="22">
         <f>IF('Modelo'!$C$33=0,"inalcanzable",$B35/'Modelo'!$C$33)</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="34">
+      <c r="B42" s="35">
         <f>$B36</f>
         <v/>
       </c>
-      <c r="C42" s="21">
+      <c r="C42" s="22">
         <f>IF('Modelo'!$C$33=0,"inalcanzable",$B36/'Modelo'!$C$33)</f>
         <v/>
       </c>
@@ -9604,19 +9929,19 @@
       </c>
     </row>
     <row r="45">
-      <c r="C45" s="35" t="n">
+      <c r="C45" s="36" t="n">
         <v>1.5</v>
       </c>
-      <c r="D45" s="35" t="n">
+      <c r="D45" s="36" t="n">
         <v>2</v>
       </c>
-      <c r="E45" s="35" t="n">
+      <c r="E45" s="36" t="n">
         <v>2.5</v>
       </c>
-      <c r="F45" s="35" t="n">
+      <c r="F45" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="G45" s="35" t="n">
+      <c r="G45" s="36" t="n">
         <v>4</v>
       </c>
     </row>
@@ -9696,15 +10021,15 @@
           <t>actual</t>
         </is>
       </c>
-      <c r="C53" s="19">
+      <c r="C53" s="20">
         <f>'Supuestos'!$C$8*1.0</f>
         <v/>
       </c>
-      <c r="D53" s="26">
+      <c r="D53" s="27">
         <f>IF(C53=0,0,('Supuestos'!$C$8*'Modelo'!$C$43+1.3*(C53-'Supuestos'!$C$8))/C53)</f>
         <v/>
       </c>
-      <c r="E53" s="19">
+      <c r="E53" s="20">
         <f>C53*(D53-1)</f>
         <v/>
       </c>
@@ -9715,15 +10040,15 @@
           <t>× 1.25</t>
         </is>
       </c>
-      <c r="C54" s="19">
+      <c r="C54" s="20">
         <f>'Supuestos'!$C$8*1.25</f>
         <v/>
       </c>
-      <c r="D54" s="26">
+      <c r="D54" s="27">
         <f>IF(C54=0,0,('Supuestos'!$C$8*'Modelo'!$C$43+1.3*(C54-'Supuestos'!$C$8))/C54)</f>
         <v/>
       </c>
-      <c r="E54" s="19">
+      <c r="E54" s="20">
         <f>C54*(D54-1)</f>
         <v/>
       </c>
@@ -9734,15 +10059,15 @@
           <t>× 1.5</t>
         </is>
       </c>
-      <c r="C55" s="19">
+      <c r="C55" s="20">
         <f>'Supuestos'!$C$8*1.5</f>
         <v/>
       </c>
-      <c r="D55" s="26">
+      <c r="D55" s="27">
         <f>IF(C55=0,0,('Supuestos'!$C$8*'Modelo'!$C$43+1.3*(C55-'Supuestos'!$C$8))/C55)</f>
         <v/>
       </c>
-      <c r="E55" s="19">
+      <c r="E55" s="20">
         <f>C55*(D55-1)</f>
         <v/>
       </c>
@@ -9753,15 +10078,15 @@
           <t>× 2</t>
         </is>
       </c>
-      <c r="C56" s="19">
+      <c r="C56" s="20">
         <f>'Supuestos'!$C$8*2.0</f>
         <v/>
       </c>
-      <c r="D56" s="26">
+      <c r="D56" s="27">
         <f>IF(C56=0,0,('Supuestos'!$C$8*'Modelo'!$C$43+1.3*(C56-'Supuestos'!$C$8))/C56)</f>
         <v/>
       </c>
-      <c r="E56" s="19">
+      <c r="E56" s="20">
         <f>C56*(D56-1)</f>
         <v/>
       </c>
@@ -9772,15 +10097,15 @@
           <t>× 3</t>
         </is>
       </c>
-      <c r="C57" s="19">
+      <c r="C57" s="20">
         <f>'Supuestos'!$C$8*3.0</f>
         <v/>
       </c>
-      <c r="D57" s="26">
+      <c r="D57" s="27">
         <f>IF(C57=0,0,('Supuestos'!$C$8*'Modelo'!$C$43+1.3*(C57-'Supuestos'!$C$8))/C57)</f>
         <v/>
       </c>
-      <c r="E57" s="19">
+      <c r="E57" s="20">
         <f>C57*(D57-1)</f>
         <v/>
       </c>
@@ -9915,19 +10240,19 @@
           <t>−10 %</t>
         </is>
       </c>
-      <c r="D7" s="19">
+      <c r="D7" s="20">
         <f>((((((((IF((('Supuestos'!$C$9*0.9))=0,0,'Supuestos'!$C$8/(('Supuestos'!$C$9*0.9))))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF((('Supuestos'!$C$9*0.9))=0,0,'Supuestos'!$C$8/(('Supuestos'!$C$9*0.9))))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF((('Supuestos'!$C$9*0.9))=0,0,'Supuestos'!$C$8/(('Supuestos'!$C$9*0.9))))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF((('Supuestos'!$C$9*0.9))=0,0,'Supuestos'!$C$8/(('Supuestos'!$C$9*0.9))))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF((('Supuestos'!$C$9*0.9))=0,0,'Supuestos'!$C$8/(('Supuestos'!$C$9*0.9))))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF((('Supuestos'!$C$9*0.9))=0,0,'Supuestos'!$C$8/(('Supuestos'!$C$9*0.9))))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF((('Supuestos'!$C$9*0.9))=0,0,'Supuestos'!$C$8/(('Supuestos'!$C$9*0.9))))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF((('Supuestos'!$C$9*0.9))=0,0,'Supuestos'!$C$8/(('Supuestos'!$C$9*0.9))))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF((('Supuestos'!$C$9*0.9))=0,0,'Supuestos'!$C$8/(('Supuestos'!$C$9*0.9))))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="E7" s="19">
+      <c r="E7" s="20">
         <f>D7-$D$6</f>
         <v/>
       </c>
-      <c r="F7" s="23">
+      <c r="F7" s="24">
         <f>IF($D$6=0,0,E7/ABS($D$6))</f>
         <v/>
       </c>
-      <c r="G7" s="21">
+      <c r="G7" s="22">
         <f>RANK(E7,$E$7:$E$14)</f>
         <v/>
       </c>
@@ -9943,19 +10268,19 @@
           <t>+10 %</t>
         </is>
       </c>
-      <c r="D8" s="19">
+      <c r="D8" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*('Supuestos'!$C$12*1.1))*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*('Supuestos'!$C$12*1.1))*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*('Supuestos'!$C$12*1.1))*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*('Supuestos'!$C$12*1.1))*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*('Supuestos'!$C$12*1.1))*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*('Supuestos'!$C$12*1.1))*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*('Supuestos'!$C$12*1.1))*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*('Supuestos'!$C$12*1.1))*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="E8" s="19">
+      <c r="E8" s="20">
         <f>D8-$D$6</f>
         <v/>
       </c>
-      <c r="F8" s="23">
+      <c r="F8" s="24">
         <f>IF($D$6=0,0,E8/ABS($D$6))</f>
         <v/>
       </c>
-      <c r="G8" s="21">
+      <c r="G8" s="22">
         <f>RANK(E8,$E$7:$E$14)</f>
         <v/>
       </c>
@@ -9971,19 +10296,19 @@
           <t>+10 %</t>
         </is>
       </c>
-      <c r="D9" s="19">
+      <c r="D9" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*('Supuestos'!$C$13*1.1))*'Supuestos'!$C$16)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*('Supuestos'!$C$13*1.1))*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*('Supuestos'!$C$13*1.1))*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*('Supuestos'!$C$13*1.1))*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*('Supuestos'!$C$13*1.1))*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*('Supuestos'!$C$13*1.1))*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*('Supuestos'!$C$13*1.1))*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*('Supuestos'!$C$13*1.1))*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="E9" s="19">
+      <c r="E9" s="20">
         <f>D9-$D$6</f>
         <v/>
       </c>
-      <c r="F9" s="23">
+      <c r="F9" s="24">
         <f>IF($D$6=0,0,E9/ABS($D$6))</f>
         <v/>
       </c>
-      <c r="G9" s="21">
+      <c r="G9" s="22">
         <f>RANK(E9,$E$7:$E$14)</f>
         <v/>
       </c>
@@ -9999,19 +10324,19 @@
           <t>+10 %</t>
         </is>
       </c>
-      <c r="D10" s="19">
+      <c r="D10" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*('Supuestos'!$C$16*1.1))+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="E10" s="19">
+      <c r="E10" s="20">
         <f>D10-$D$6</f>
         <v/>
       </c>
-      <c r="F10" s="23">
+      <c r="F10" s="24">
         <f>IF($D$6=0,0,E10/ABS($D$6))</f>
         <v/>
       </c>
-      <c r="G10" s="21">
+      <c r="G10" s="22">
         <f>RANK(E10,$E$7:$E$14)</f>
         <v/>
       </c>
@@ -10027,19 +10352,19 @@
           <t>+10 %</t>
         </is>
       </c>
-      <c r="D11" s="19">
+      <c r="D11" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*('Supuestos'!$C$18*1.1))*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="E11" s="19">
+      <c r="E11" s="20">
         <f>D11-$D$6</f>
         <v/>
       </c>
-      <c r="F11" s="23">
+      <c r="F11" s="24">
         <f>IF($D$6=0,0,E11/ABS($D$6))</f>
         <v/>
       </c>
-      <c r="G11" s="21">
+      <c r="G11" s="22">
         <f>RANK(E11,$E$7:$E$14)</f>
         <v/>
       </c>
@@ -10055,19 +10380,19 @@
           <t>+10 %</t>
         </is>
       </c>
-      <c r="D12" s="19">
+      <c r="D12" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*('Supuestos'!$C$22*1.1))*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="E12" s="19">
+      <c r="E12" s="20">
         <f>D12-$D$6</f>
         <v/>
       </c>
-      <c r="F12" s="23">
+      <c r="F12" s="24">
         <f>IF($D$6=0,0,E12/ABS($D$6))</f>
         <v/>
       </c>
-      <c r="G12" s="21">
+      <c r="G12" s="22">
         <f>RANK(E12,$E$7:$E$14)</f>
         <v/>
       </c>
@@ -10083,19 +10408,19 @@
           <t>+10 %</t>
         </is>
       </c>
-      <c r="D13" s="19">
+      <c r="D13" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*('Supuestos'!$C$30*1.1))*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-'Supuestos'!$C$35))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="E13" s="19">
+      <c r="E13" s="20">
         <f>D13-$D$6</f>
         <v/>
       </c>
-      <c r="F13" s="23">
+      <c r="F13" s="24">
         <f>IF($D$6=0,0,E13/ABS($D$6))</f>
         <v/>
       </c>
-      <c r="G13" s="21">
+      <c r="G13" s="22">
         <f>RANK(E13,$E$7:$E$14)</f>
         <v/>
       </c>
@@ -10111,19 +10436,19 @@
           <t>−10 %</t>
         </is>
       </c>
-      <c r="D14" s="19">
+      <c r="D14" s="20">
         <f>((((((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$16)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$18)*'Supuestos'!$C$17)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$20)*'Supuestos'!$C$19)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$22)*'Supuestos'!$C$21)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$24)*'Supuestos'!$C$23)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$26)*'Supuestos'!$C$25)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$28)*'Supuestos'!$C$27)+(((((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$12)*'Supuestos'!$C$13)*'Supuestos'!$C$30)*'Supuestos'!$C$29))*('Supuestos'!$C$40+'Supuestos'!$C$41+'Supuestos'!$C$42))*(1-'Supuestos'!$C$33-'Supuestos'!$C$34-('Supuestos'!$C$35*0.9)))-((IF(('Supuestos'!$C$9)=0,0,'Supuestos'!$C$8/('Supuestos'!$C$9)))*'Supuestos'!$C$36)-'Supuestos'!$C$37-'Supuestos'!$C$8)</f>
         <v/>
       </c>
-      <c r="E14" s="19">
+      <c r="E14" s="20">
         <f>D14-$D$6</f>
         <v/>
       </c>
-      <c r="F14" s="23">
+      <c r="F14" s="24">
         <f>IF($D$6=0,0,E14/ABS($D$6))</f>
         <v/>
       </c>
-      <c r="G14" s="21">
+      <c r="G14" s="22">
         <f>RANK(E14,$E$7:$E$14)</f>
         <v/>
       </c>
@@ -10266,51 +10591,51 @@
           <t>Inversión en publicidad del mes</t>
         </is>
       </c>
-      <c r="C6" s="19">
+      <c r="C6" s="20">
         <f>'Supuestos'!$C$8*1</f>
         <v/>
       </c>
-      <c r="D6" s="19">
+      <c r="D6" s="20">
         <f>C6*(1+'Supuestos'!$C$48)</f>
         <v/>
       </c>
-      <c r="E6" s="19">
+      <c r="E6" s="20">
         <f>D6*(1+'Supuestos'!$C$48)</f>
         <v/>
       </c>
-      <c r="F6" s="19">
+      <c r="F6" s="20">
         <f>E6*(1+'Supuestos'!$C$48)</f>
         <v/>
       </c>
-      <c r="G6" s="19">
+      <c r="G6" s="20">
         <f>F6*(1+'Supuestos'!$C$48)</f>
         <v/>
       </c>
-      <c r="H6" s="19">
+      <c r="H6" s="20">
         <f>G6*(1+'Supuestos'!$C$48)</f>
         <v/>
       </c>
-      <c r="I6" s="19">
+      <c r="I6" s="20">
         <f>H6*(1+'Supuestos'!$C$48)</f>
         <v/>
       </c>
-      <c r="J6" s="19">
+      <c r="J6" s="20">
         <f>I6*(1+'Supuestos'!$C$48)</f>
         <v/>
       </c>
-      <c r="K6" s="19">
+      <c r="K6" s="20">
         <f>J6*(1+'Supuestos'!$C$48)</f>
         <v/>
       </c>
-      <c r="L6" s="19">
+      <c r="L6" s="20">
         <f>K6*(1+'Supuestos'!$C$48)</f>
         <v/>
       </c>
-      <c r="M6" s="19">
+      <c r="M6" s="20">
         <f>L6*(1+'Supuestos'!$C$48)</f>
         <v/>
       </c>
-      <c r="N6" s="19">
+      <c r="N6" s="20">
         <f>M6*(1+'Supuestos'!$C$48)</f>
         <v/>
       </c>
@@ -10325,55 +10650,55 @@
           <t>Visitas compradas</t>
         </is>
       </c>
-      <c r="C7" s="21">
+      <c r="C7" s="22">
         <f>IF('Modelo'!$C$7=0,0,C6/'Modelo'!$C$7)</f>
         <v/>
       </c>
-      <c r="D7" s="21">
+      <c r="D7" s="22">
         <f>IF('Modelo'!$C$7=0,0,D6/'Modelo'!$C$7)</f>
         <v/>
       </c>
-      <c r="E7" s="21">
+      <c r="E7" s="22">
         <f>IF('Modelo'!$C$7=0,0,E6/'Modelo'!$C$7)</f>
         <v/>
       </c>
-      <c r="F7" s="21">
+      <c r="F7" s="22">
         <f>IF('Modelo'!$C$7=0,0,F6/'Modelo'!$C$7)</f>
         <v/>
       </c>
-      <c r="G7" s="21">
+      <c r="G7" s="22">
         <f>IF('Modelo'!$C$7=0,0,G6/'Modelo'!$C$7)</f>
         <v/>
       </c>
-      <c r="H7" s="21">
+      <c r="H7" s="22">
         <f>IF('Modelo'!$C$7=0,0,H6/'Modelo'!$C$7)</f>
         <v/>
       </c>
-      <c r="I7" s="21">
+      <c r="I7" s="22">
         <f>IF('Modelo'!$C$7=0,0,I6/'Modelo'!$C$7)</f>
         <v/>
       </c>
-      <c r="J7" s="21">
+      <c r="J7" s="22">
         <f>IF('Modelo'!$C$7=0,0,J6/'Modelo'!$C$7)</f>
         <v/>
       </c>
-      <c r="K7" s="21">
+      <c r="K7" s="22">
         <f>IF('Modelo'!$C$7=0,0,K6/'Modelo'!$C$7)</f>
         <v/>
       </c>
-      <c r="L7" s="21">
+      <c r="L7" s="22">
         <f>IF('Modelo'!$C$7=0,0,L6/'Modelo'!$C$7)</f>
         <v/>
       </c>
-      <c r="M7" s="21">
+      <c r="M7" s="22">
         <f>IF('Modelo'!$C$7=0,0,M6/'Modelo'!$C$7)</f>
         <v/>
       </c>
-      <c r="N7" s="21">
+      <c r="N7" s="22">
         <f>IF('Modelo'!$C$7=0,0,N6/'Modelo'!$C$7)</f>
         <v/>
       </c>
-      <c r="O7" s="20">
+      <c r="O7" s="21">
         <f>SUM(C7:N7)</f>
         <v/>
       </c>
@@ -10384,51 +10709,51 @@
           <t>Ventas del producto principal</t>
         </is>
       </c>
-      <c r="C8" s="24">
+      <c r="C8" s="25">
         <f>C7*'Modelo'!$C$32</f>
         <v/>
       </c>
-      <c r="D8" s="24">
+      <c r="D8" s="25">
         <f>D7*'Modelo'!$C$32</f>
         <v/>
       </c>
-      <c r="E8" s="24">
+      <c r="E8" s="25">
         <f>E7*'Modelo'!$C$32</f>
         <v/>
       </c>
-      <c r="F8" s="24">
+      <c r="F8" s="25">
         <f>F7*'Modelo'!$C$32</f>
         <v/>
       </c>
-      <c r="G8" s="24">
+      <c r="G8" s="25">
         <f>G7*'Modelo'!$C$32</f>
         <v/>
       </c>
-      <c r="H8" s="24">
+      <c r="H8" s="25">
         <f>H7*'Modelo'!$C$32</f>
         <v/>
       </c>
-      <c r="I8" s="24">
+      <c r="I8" s="25">
         <f>I7*'Modelo'!$C$32</f>
         <v/>
       </c>
-      <c r="J8" s="24">
+      <c r="J8" s="25">
         <f>J7*'Modelo'!$C$32</f>
         <v/>
       </c>
-      <c r="K8" s="24">
+      <c r="K8" s="25">
         <f>K7*'Modelo'!$C$32</f>
         <v/>
       </c>
-      <c r="L8" s="24">
+      <c r="L8" s="25">
         <f>L7*'Modelo'!$C$32</f>
         <v/>
       </c>
-      <c r="M8" s="24">
+      <c r="M8" s="25">
         <f>M7*'Modelo'!$C$32</f>
         <v/>
       </c>
-      <c r="N8" s="24">
+      <c r="N8" s="25">
         <f>N7*'Modelo'!$C$32</f>
         <v/>
       </c>
@@ -10443,51 +10768,51 @@
           <t>Facturado (todos los productos)</t>
         </is>
       </c>
-      <c r="C9" s="19">
+      <c r="C9" s="20">
         <f>C7*'Modelo'!$C$33</f>
         <v/>
       </c>
-      <c r="D9" s="19">
+      <c r="D9" s="20">
         <f>D7*'Modelo'!$C$33</f>
         <v/>
       </c>
-      <c r="E9" s="19">
+      <c r="E9" s="20">
         <f>E7*'Modelo'!$C$33</f>
         <v/>
       </c>
-      <c r="F9" s="19">
+      <c r="F9" s="20">
         <f>F7*'Modelo'!$C$33</f>
         <v/>
       </c>
-      <c r="G9" s="19">
+      <c r="G9" s="20">
         <f>G7*'Modelo'!$C$33</f>
         <v/>
       </c>
-      <c r="H9" s="19">
+      <c r="H9" s="20">
         <f>H7*'Modelo'!$C$33</f>
         <v/>
       </c>
-      <c r="I9" s="19">
+      <c r="I9" s="20">
         <f>I7*'Modelo'!$C$33</f>
         <v/>
       </c>
-      <c r="J9" s="19">
+      <c r="J9" s="20">
         <f>J7*'Modelo'!$C$33</f>
         <v/>
       </c>
-      <c r="K9" s="19">
+      <c r="K9" s="20">
         <f>K7*'Modelo'!$C$33</f>
         <v/>
       </c>
-      <c r="L9" s="19">
+      <c r="L9" s="20">
         <f>L7*'Modelo'!$C$33</f>
         <v/>
       </c>
-      <c r="M9" s="19">
+      <c r="M9" s="20">
         <f>M7*'Modelo'!$C$33</f>
         <v/>
       </c>
-      <c r="N9" s="19">
+      <c r="N9" s="20">
         <f>N7*'Modelo'!$C$33</f>
         <v/>
       </c>
@@ -10502,51 +10827,51 @@
           <t>Cash cobrado en el mes</t>
         </is>
       </c>
-      <c r="C10" s="19">
+      <c r="C10" s="20">
         <f>C9*'Supuestos'!$C$40</f>
         <v/>
       </c>
-      <c r="D10" s="19">
+      <c r="D10" s="20">
         <f>D9*'Supuestos'!$C$40+C9*'Supuestos'!$C$41</f>
         <v/>
       </c>
-      <c r="E10" s="19">
+      <c r="E10" s="20">
         <f>E9*'Supuestos'!$C$40+D9*'Supuestos'!$C$41+C9*'Supuestos'!$C$42</f>
         <v/>
       </c>
-      <c r="F10" s="19">
+      <c r="F10" s="20">
         <f>F9*'Supuestos'!$C$40+E9*'Supuestos'!$C$41+D9*'Supuestos'!$C$42</f>
         <v/>
       </c>
-      <c r="G10" s="19">
+      <c r="G10" s="20">
         <f>G9*'Supuestos'!$C$40+F9*'Supuestos'!$C$41+E9*'Supuestos'!$C$42</f>
         <v/>
       </c>
-      <c r="H10" s="19">
+      <c r="H10" s="20">
         <f>H9*'Supuestos'!$C$40+G9*'Supuestos'!$C$41+F9*'Supuestos'!$C$42</f>
         <v/>
       </c>
-      <c r="I10" s="19">
+      <c r="I10" s="20">
         <f>I9*'Supuestos'!$C$40+H9*'Supuestos'!$C$41+G9*'Supuestos'!$C$42</f>
         <v/>
       </c>
-      <c r="J10" s="19">
+      <c r="J10" s="20">
         <f>J9*'Supuestos'!$C$40+I9*'Supuestos'!$C$41+H9*'Supuestos'!$C$42</f>
         <v/>
       </c>
-      <c r="K10" s="19">
+      <c r="K10" s="20">
         <f>K9*'Supuestos'!$C$40+J9*'Supuestos'!$C$41+I9*'Supuestos'!$C$42</f>
         <v/>
       </c>
-      <c r="L10" s="19">
+      <c r="L10" s="20">
         <f>L9*'Supuestos'!$C$40+K9*'Supuestos'!$C$41+J9*'Supuestos'!$C$42</f>
         <v/>
       </c>
-      <c r="M10" s="19">
+      <c r="M10" s="20">
         <f>M9*'Supuestos'!$C$40+L9*'Supuestos'!$C$41+K9*'Supuestos'!$C$42</f>
         <v/>
       </c>
-      <c r="N10" s="19">
+      <c r="N10" s="20">
         <f>N9*'Supuestos'!$C$40+M9*'Supuestos'!$C$41+L9*'Supuestos'!$C$42</f>
         <v/>
       </c>
@@ -10561,51 +10886,51 @@
           <t>Comisiones y reembolsos</t>
         </is>
       </c>
-      <c r="C11" s="19">
+      <c r="C11" s="20">
         <f>C10*('Supuestos'!$C$33+'Supuestos'!$C$34+'Supuestos'!$C$35)</f>
         <v/>
       </c>
-      <c r="D11" s="19">
+      <c r="D11" s="20">
         <f>D10*('Supuestos'!$C$33+'Supuestos'!$C$34+'Supuestos'!$C$35)</f>
         <v/>
       </c>
-      <c r="E11" s="19">
+      <c r="E11" s="20">
         <f>E10*('Supuestos'!$C$33+'Supuestos'!$C$34+'Supuestos'!$C$35)</f>
         <v/>
       </c>
-      <c r="F11" s="19">
+      <c r="F11" s="20">
         <f>F10*('Supuestos'!$C$33+'Supuestos'!$C$34+'Supuestos'!$C$35)</f>
         <v/>
       </c>
-      <c r="G11" s="19">
+      <c r="G11" s="20">
         <f>G10*('Supuestos'!$C$33+'Supuestos'!$C$34+'Supuestos'!$C$35)</f>
         <v/>
       </c>
-      <c r="H11" s="19">
+      <c r="H11" s="20">
         <f>H10*('Supuestos'!$C$33+'Supuestos'!$C$34+'Supuestos'!$C$35)</f>
         <v/>
       </c>
-      <c r="I11" s="19">
+      <c r="I11" s="20">
         <f>I10*('Supuestos'!$C$33+'Supuestos'!$C$34+'Supuestos'!$C$35)</f>
         <v/>
       </c>
-      <c r="J11" s="19">
+      <c r="J11" s="20">
         <f>J10*('Supuestos'!$C$33+'Supuestos'!$C$34+'Supuestos'!$C$35)</f>
         <v/>
       </c>
-      <c r="K11" s="19">
+      <c r="K11" s="20">
         <f>K10*('Supuestos'!$C$33+'Supuestos'!$C$34+'Supuestos'!$C$35)</f>
         <v/>
       </c>
-      <c r="L11" s="19">
+      <c r="L11" s="20">
         <f>L10*('Supuestos'!$C$33+'Supuestos'!$C$34+'Supuestos'!$C$35)</f>
         <v/>
       </c>
-      <c r="M11" s="19">
+      <c r="M11" s="20">
         <f>M10*('Supuestos'!$C$33+'Supuestos'!$C$34+'Supuestos'!$C$35)</f>
         <v/>
       </c>
-      <c r="N11" s="19">
+      <c r="N11" s="20">
         <f>N10*('Supuestos'!$C$33+'Supuestos'!$C$34+'Supuestos'!$C$35)</f>
         <v/>
       </c>
@@ -10620,51 +10945,51 @@
           <t>Costos por unidad (herramientas, WhatsApp, IA)</t>
         </is>
       </c>
-      <c r="C12" s="19">
+      <c r="C12" s="20">
         <f>C7*'Supuestos'!$C$36</f>
         <v/>
       </c>
-      <c r="D12" s="19">
+      <c r="D12" s="20">
         <f>D7*'Supuestos'!$C$36</f>
         <v/>
       </c>
-      <c r="E12" s="19">
+      <c r="E12" s="20">
         <f>E7*'Supuestos'!$C$36</f>
         <v/>
       </c>
-      <c r="F12" s="19">
+      <c r="F12" s="20">
         <f>F7*'Supuestos'!$C$36</f>
         <v/>
       </c>
-      <c r="G12" s="19">
+      <c r="G12" s="20">
         <f>G7*'Supuestos'!$C$36</f>
         <v/>
       </c>
-      <c r="H12" s="19">
+      <c r="H12" s="20">
         <f>H7*'Supuestos'!$C$36</f>
         <v/>
       </c>
-      <c r="I12" s="19">
+      <c r="I12" s="20">
         <f>I7*'Supuestos'!$C$36</f>
         <v/>
       </c>
-      <c r="J12" s="19">
+      <c r="J12" s="20">
         <f>J7*'Supuestos'!$C$36</f>
         <v/>
       </c>
-      <c r="K12" s="19">
+      <c r="K12" s="20">
         <f>K7*'Supuestos'!$C$36</f>
         <v/>
       </c>
-      <c r="L12" s="19">
+      <c r="L12" s="20">
         <f>L7*'Supuestos'!$C$36</f>
         <v/>
       </c>
-      <c r="M12" s="19">
+      <c r="M12" s="20">
         <f>M7*'Supuestos'!$C$36</f>
         <v/>
       </c>
-      <c r="N12" s="19">
+      <c r="N12" s="20">
         <f>N7*'Supuestos'!$C$36</f>
         <v/>
       </c>
@@ -10679,51 +11004,51 @@
           <t>Costos fijos del mes</t>
         </is>
       </c>
-      <c r="C13" s="19">
+      <c r="C13" s="20">
         <f>'Supuestos'!$C$37*1</f>
         <v/>
       </c>
-      <c r="D13" s="19">
+      <c r="D13" s="20">
         <f>'Supuestos'!$C$37*1</f>
         <v/>
       </c>
-      <c r="E13" s="19">
+      <c r="E13" s="20">
         <f>'Supuestos'!$C$37*1</f>
         <v/>
       </c>
-      <c r="F13" s="19">
+      <c r="F13" s="20">
         <f>'Supuestos'!$C$37*1</f>
         <v/>
       </c>
-      <c r="G13" s="19">
+      <c r="G13" s="20">
         <f>'Supuestos'!$C$37*1</f>
         <v/>
       </c>
-      <c r="H13" s="19">
+      <c r="H13" s="20">
         <f>'Supuestos'!$C$37*1</f>
         <v/>
       </c>
-      <c r="I13" s="19">
+      <c r="I13" s="20">
         <f>'Supuestos'!$C$37*1</f>
         <v/>
       </c>
-      <c r="J13" s="19">
+      <c r="J13" s="20">
         <f>'Supuestos'!$C$37*1</f>
         <v/>
       </c>
-      <c r="K13" s="19">
+      <c r="K13" s="20">
         <f>'Supuestos'!$C$37*1</f>
         <v/>
       </c>
-      <c r="L13" s="19">
+      <c r="L13" s="20">
         <f>'Supuestos'!$C$37*1</f>
         <v/>
       </c>
-      <c r="M13" s="19">
+      <c r="M13" s="20">
         <f>'Supuestos'!$C$37*1</f>
         <v/>
       </c>
-      <c r="N13" s="19">
+      <c r="N13" s="20">
         <f>'Supuestos'!$C$37*1</f>
         <v/>
       </c>
@@ -10852,51 +11177,51 @@
           <t>Saldo de caja (caja inicial + ganancia acumulada)</t>
         </is>
       </c>
-      <c r="C16" s="19">
+      <c r="C16" s="20">
         <f>'Supuestos'!$C$49+C15</f>
         <v/>
       </c>
-      <c r="D16" s="19">
+      <c r="D16" s="20">
         <f>'Supuestos'!$C$49+D15</f>
         <v/>
       </c>
-      <c r="E16" s="19">
+      <c r="E16" s="20">
         <f>'Supuestos'!$C$49+E15</f>
         <v/>
       </c>
-      <c r="F16" s="19">
+      <c r="F16" s="20">
         <f>'Supuestos'!$C$49+F15</f>
         <v/>
       </c>
-      <c r="G16" s="19">
+      <c r="G16" s="20">
         <f>'Supuestos'!$C$49+G15</f>
         <v/>
       </c>
-      <c r="H16" s="19">
+      <c r="H16" s="20">
         <f>'Supuestos'!$C$49+H15</f>
         <v/>
       </c>
-      <c r="I16" s="19">
+      <c r="I16" s="20">
         <f>'Supuestos'!$C$49+I15</f>
         <v/>
       </c>
-      <c r="J16" s="19">
+      <c r="J16" s="20">
         <f>'Supuestos'!$C$49+J15</f>
         <v/>
       </c>
-      <c r="K16" s="19">
+      <c r="K16" s="20">
         <f>'Supuestos'!$C$49+K15</f>
         <v/>
       </c>
-      <c r="L16" s="19">
+      <c r="L16" s="20">
         <f>'Supuestos'!$C$49+L15</f>
         <v/>
       </c>
-      <c r="M16" s="19">
+      <c r="M16" s="20">
         <f>'Supuestos'!$C$49+M15</f>
         <v/>
       </c>
-      <c r="N16" s="19">
+      <c r="N16" s="20">
         <f>'Supuestos'!$C$49+N15</f>
         <v/>
       </c>

</xml_diff>